<commit_message>
dashboard: regenerate captures against the two real clients
The committed screenshots and documents predated the client work: they showed
one test client with a two-market scope, and the documents carried the
fixture-written assessments that are now gone.

Regenerated by the full gate. The document set is now Simtec at 29 projects
and JKR at 149, both against their real stored scopes, and the by-market
sections carry the truncation note where the 25-per-market cap bites.

The only change in screens-audit.json is Clients rows 1 -> 2, which is JKR
arriving. The five ok:false entries in that file are byte-identical to the
previous run and are a harness expectation rather than a defect: Records,
Legacy pipeline and Legacy GLI have no h1 element at all, and the "Clients
detail" case is pointed at /clients rather than at a client. All five report
zero console errors, zero page errors and zero failed requests.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/e2e/shots/documents/full-report.xlsx
+++ b/dashboard/e2e/shots/documents/full-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="110">
   <si>
     <t>Market intelligence report</t>
   </si>
@@ -19,16 +19,16 @@
     <t>Prepared for Simtec Attractions by Philip Kwong</t>
   </si>
   <si>
-    <t>Geography: Clark County, Las Vegas</t>
+    <t>Geography: Altamonte Springs, Anaheim, Atlanta, Bonita Springs, Central Florida Tourism Oversight District, Clark County, Kissimmee, Lake Buena Vista, Las Vegas, Miami-Dade County, Nashville, Oakland, Phoenix, San Antonio, South Florida, Walt Disney World</t>
   </si>
   <si>
     <t>Period: July 2026</t>
   </si>
   <si>
-    <t>Filters: dormant excluded | context records included | stage: filed</t>
-  </si>
-  <si>
-    <t>Basis: 44 projects, 76 records</t>
+    <t>Filters: dormant excluded | context records included | stage: hearing scheduled | stage: approved | stage: permitted | stage: under construction | venue: Theme Park | venue: Amusement Park | venue: Waterpark | venue: Family Entertainment Center | venue: Museum | venue: Aquarium | venue: Science Center | venue: Heritage/Cultural Site | venue: Arena/Stadium | venue: Integrated Resort | venue: Casino/Gaming | venue: Entertainment District | venue: Leisure Destination | venue: Mixed-Use Development</t>
+  </si>
+  <si>
+    <t>Basis: 29 projects, 86 records</t>
   </si>
   <si>
     <t>Section</t>
@@ -52,397 +52,290 @@
     <t>ASSESSMENT</t>
   </si>
   <si>
-    <t>This report covers Clark County, Las Vegas for July 2026. It is drawn from 44 projects and 76 captured records. Anything outside that geography or period is not covered here.</t>
+    <t>This report covers Altamonte Springs, Anaheim, Atlanta, Bonita Springs, Central Florida Tourism Oversight District, Clark County, Kissimmee, Lake Buena Vista, Las Vegas, Miami-Dade County, Nashville, Oakland, Phoenix, San Antonio, South Florida, Walt Disney World for July 2026. It is drawn from 29 projects and 86 captured records. Anything outside that geography or period is not covered here.</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
+    <t>What moved</t>
+  </si>
+  <si>
+    <t>RECORD</t>
+  </si>
+  <si>
+    <t>OCVibe: filed to approved</t>
+  </si>
+  <si>
+    <t>2026-07-13 | Anaheim</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3646#item-heb30443bfb8b</t>
+  </si>
+  <si>
     <t>Headline finds</t>
   </si>
   <si>
-    <t>RECORD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nevada Palace resort: PA-26-700023-NEVADA PALACE, LLC:
-PLAN AMENDMENT to redesignate the existing land use category from Entertainment Mixed-Use (EM) to Compact Neighborhood (CN) on 29.46 acres. Generally located northeast of Boulder Highway and southeast of Harmon Avenue within Sunrise Manor and Whitney. JG/gc (For possible action)</t>
-  </si>
-  <si>
-    <t>2026-08-04 | Clark County</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/Legislation.aspx#matter-110561</t>
+    <t>OCVibe: 4. Determinar sobre la base de la evidencia presentada por Anaheim Real Estate Partners, LLC, TS Anaheim, LLC y FCD, LLC (OCVIBE), que el propietario de la propiedad ha cumplido de buena fe con los té</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_7f2f654f7555addc70231de198fa22d9.pdf&amp;view=1#item-h9f002fc7dbca</t>
   </si>
   <si>
     <t>PRESS</t>
   </si>
   <si>
-    <t>Top Gun Las Vegas: Top Gun Vegas Locks South Strip Site at 4815 Las Vegas ...</t>
-  </si>
-  <si>
-    <t>2026-07-26 | Las Vegas</t>
-  </si>
-  <si>
-    <t>https://deeparrival.com/news/top-gun-vegas-south-strip-site-july-2026/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Southern Highlands Golf Club leisure development: UC-26-0350-SOUTHERN HIGHLANDS GOLF CLUB:
-USE PERMITS for the following: 1) multi-family residential development; 2) modified development standards.
-DESIGN REVIEW for a multi-family residential development in conjunction with an existing golf course on a 1.7 acre portion of 8.05 acres in a C-2 (General Commercial District) Zone within the Southern Highlands Planned Community (PCO) Overlay.  Generally located north of Robert Trent Jones Lane and west of Southern Highlands Parkway within Enterprise.  JJ/bb/kh  (For possible action)</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/Legislation.aspx#matter-110519</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visible Noise family entertainment centre: UC-26-0303-VISIBLE NOISE, LLC:
-HOLDOVER USE PERMIT for a proposed recreational or entertainment facility within an existing office/warehouse complex on a portion of 5.31 acres in an IP (Industrial Park) Zone within the Airport Environs (AE-60) Overlay. Generally located west of Tenaya Way and north of Sunset Road within Spring Valley.  MN/rp/cv  (For possible action)</t>
-  </si>
-  <si>
-    <t>2026-08-03 | Clark County</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/Legislation.aspx#matter-110501</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tropicana Land resort: WS-26-0113-TROPICANA LAND, LLC:
-HOLDOVER WAIVER OF DEVELOPMENT STANDARDS for modified driveway geometrics.
-DESIGN REVIEW for a resort hotel on a 26.11 acre portion of 35.11 acres in a CR (Commercial Resort) Zone within the Airport Environs (AE-60) Overlay. Generally located south of Tropicana Avenue and east of Las Vegas Boulevard South within Paradise.  JG/nm/kh  (For possible action)</t>
+    <t>Heart Hotel / Kulik River: Las Vegas Topic Kulik River Capital</t>
+  </si>
+  <si>
+    <t>2026-07-24 | Clark County</t>
+  </si>
+  <si>
+    <t>https://news3lv.com/topic/Kulik%20River%20Capital</t>
+  </si>
+  <si>
+    <t>CFTOD / Walt Disney World: Approve the District Administrator to execute a Non-exclusive temporary easement with permanent easement to Walt Disney Parks &amp; Resorts, U.S. Inc for underground communication lines</t>
+  </si>
+  <si>
+    <t>2026-01-23 | Central Florida Tourism Oversight District</t>
+  </si>
+  <si>
+    <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/1-23-2026-BOS-Agenda-Packet-FINALcs.pdf#item-6.4-p146</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weston Urban leisure development: Discussion and possible action to authorize execution of a Master Economic Incentive Agreement between Weston Urban, LLC and the City of San Antonio as a source of funding for public improvements related to the redevelopment of the property located at 322 W. Commerce, for an amount up to $250,000.
+</t>
+  </si>
+  <si>
+    <t>2021-09-20 | San Antonio</t>
+  </si>
+  <si>
+    <t>https://sanantonio.legistar.com/gateway.aspx?M=l&amp;ID=43966</t>
+  </si>
+  <si>
+    <t>World Buddhism Association Headquarters &amp; MGM-Grand Bally's integrated resort: 4. AR-26-400041 (UC-25-0544)-WORLD BUDDHISM ASSOCIATION HEADQUARTERS &amp; MGM-GRAND BALLY'S, LLC LEASE: USE PERMIT FIRST APPLICATION FOR REVIEW for a recreational or entertainment facility. DESIGN REVIEW</t>
+  </si>
+  <si>
+    <t>2026-07-14 | Clark County</t>
+  </si>
+  <si>
+    <t>https://www.clarkcountynv.gov/adobe/assets/urn:aaid:aem:35f66646-63c2-45e2-8052-2833536974fb/original/as/Winchester-Agenda-071426.pdf#item-ar-26-400041+uc-25-0544</t>
+  </si>
+  <si>
+    <t>Toll South LV leisure development: ORD-26-900159: Conduct a public hearing on an ordinance to consider adoption of a Development Agreement with Toll South LV LLC for a single-family residential subdivision on 0.89 acres, generally located east of Hinson Street and north of Silverado Ranch Boulevard within Enterprise. JJ/tpd (For possible action)</t>
   </si>
   <si>
     <t>2026-07-21 | Clark County</t>
   </si>
   <si>
-    <t>https://clark.legistar.com/Legislation.aspx#matter-110434</t>
-  </si>
-  <si>
-    <t>multifamily and mixed-use development that includes a residential component as: 40. Bill No. 2026-16 - For possible action - Authorizes multifamily and mixed-use development that includes a residential component as a conditional use on property zoned for commercial use, in accord</t>
-  </si>
-  <si>
-    <t>2026-05-20 | Las Vegas</t>
-  </si>
-  <si>
-    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=42386#item-ha228cfd5c1c1</t>
-  </si>
-  <si>
-    <t>163 At Casino Drive casino: Approve and authorize the Chair to sign Supplemental No. 8 to the interlocal contract between Clark County and Regional Flood Control District to extend the contract term for design of the State Route 163 at Casino Drive project.  (For possible action)</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110472</t>
-  </si>
-  <si>
-    <t xml:space="preserve">South Decatur Holding CO leisure development: PA-26-700010-SOUTH DECATUR HOLDING CO., LLC:
-PLAN AMENDMENT to redesignate the existing land use category from Neighborhood Commercial (NC) to Compact Neighborhood (CN) on 2.64 acres.  Generally located east of Decatur Boulevard and south of Moberly Avenue (alignment) within Enterprise. MN/rk (For possible action)</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110447</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G D Carden Entertainment museum: ET-26-400054 (UC-25-0072)-GD CARDEN ENTERTAINMENT, LLC:
-USE PERMITS FIRST EXTENSION OF TIME for the following: 1) recreational or entertainment facility; 2) museum; and 3) live entertainment. 
-WAIVERS OF DEVELOPMENT STANDARDS for the following: 1) eliminate and reduce setbacks; 2) reduce parking requirements; 3) waive full off-site improvements; 4) reduce driveway approach distance; 5) reduce driveway departure distance; and 6) reduce driveway width.
-DESIGN REVIEW for a recreational or entertainment facility and museum on 1.82 acres in an RS20 (Residential Single-Family 20) Zone within a Historic Designation (HDO) Overlay.  Generally located north of Vegas Drive and west of Valley Drive within the Lone Mountain Planning Area.  WM/rr/cv  (For possible action)</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110423</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shamaim Henderson family entertainment centre: UC-26-0309-SHAMAIM HENDERSON, LLC:
-USE PERMITS for the following: 1) an avocational or vocational training facility; and 2) a recreational or entertainment facility on a portion of 5.11 acres in an IL (Industrial Light) Zone and an IP (Industrial Park) Zone within the Airport Environs (AE-60 &amp; AE-65) Overlay. Generally located south of Pilot Road and west of Bermuda Road within Enterprise.  MN/hw/cv  (For possible action)</t>
-  </si>
-  <si>
-    <t>2026-07-20 | Clark County</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110386</t>
+    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110431</t>
+  </si>
+  <si>
+    <t>BDA South leisure development: ORD-26-900280: Conduct a public hearing on an ordinance to consider adoption of a Development Agreement with BDA South, LLC for a vehicle wash on 1.08 acres, generally located north of Wigwam Avenue and east of Arville Street within Enterprise. JJ/tpd (For possible action)</t>
+  </si>
+  <si>
+    <t>https://clark.legistar.com/Legislation.aspx#matter-110432</t>
+  </si>
+  <si>
+    <t>12802 Old Hickory Boulevard mixed-use development: An ordinance to amend Title 17 of the Metropolitan Code of Laws, the Zoning Ordinance of The Metropolitan Government of Nashville and Davidson County, by changing from AR2a to SP zoning for property located at 12802 Old Hickory Boulevard, approximately 148 feet southwest of Logistics Way (3.6 acres), to permit a mixed use development, all of which is described herein (Proposal No. 2026SP-025-001).</t>
+  </si>
+  <si>
+    <t>2026-08-03 | Nashville</t>
+  </si>
+  <si>
+    <t>https://nashville.legistar.com/gateway.aspx?M=l&amp;ID=20788</t>
+  </si>
+  <si>
+    <t>to authorize building material restrictions and requirements for BL2026-1474: An ordinance to amend Title 17 of the Metropolitan Code of Laws, the Zoning Ordinance of The Metropolitan Government of Nashville and Davidson County, by changing from IR to SP zoning for property located at 1205 2nd Avenue North, approximately 129 feet north of Madison Street (0.46 acres), to permit a mixed use development, all of which is described herein (Proposal No. 2026SP-024-001).</t>
+  </si>
+  <si>
+    <t>https://nashville.legistar.com/gateway.aspx?M=l&amp;ID=20782</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mirage Propco casino: DR-26-0313-MIRAGE PROPCO, LLC:
+DESIGN REVIEW for a proposed theater expansion in conjunction with a previously approved resort hotel (Hard Rock Hotel &amp; Casino) on a portion of 76.93 acres in a CR (Commercial Resort) Zone. Generally located west of Las Vegas Boulevard South and south of Spring Mountain Road within Paradise.  TS/hw/cv  (For possible action)</t>
+  </si>
+  <si>
+    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110419</t>
   </si>
   <si>
     <t>By market</t>
   </si>
   <si>
-    <t>Clark County | LV Warm Springs by its General Partner LV Warm Springs LV leisure development: ORD-26-900492: Introduce an ordinance to consider adoption of a Development Agreement with LV Warm Springs by its’ General Partner LV Warm Springs  LV Warm Springs CP LLC by Flex GP holding Corp Owner for a warehouse and distribution center on 6.47 acres, generally located west of Tenaya Way and south of Arby Avenue within Spring Valley. MN/rp (For possible action)</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/Legislation.aspx#matter-110572</t>
-  </si>
-  <si>
-    <t>Clark County | HD Oleta leisure development: ORD-26-900429: Introduce an ordinance to consider adoption of a Development Agreement with HD OLETA LLC and LAS VEGAS PAVING CORP for an office/warehouse complex on 9.67 acres, generally located south of Oleta Avenue and west of Jones Boulevard within Enterprise. JJ/tpd (For possible action)</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/Legislation.aspx#matter-110571</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | Nevada Palace resort: PA-26-700023-NEVADA PALACE, LLC:
-PLAN AMENDMENT to redesignate the existing land use category from Entertainment Mixed-Use (EM) to Compact Neighborhood (CN) on 29.46 acres. Generally located northeast of Boulder Highway and southeast of Harmon Avenue within Sunrise Manor and Whitney. JG/gc (For possible action)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | Southern Highlands Golf Club leisure development: UC-26-0350-SOUTHERN HIGHLANDS GOLF CLUB:
-USE PERMITS for the following: 1) multi-family residential development; 2) modified development standards.
-DESIGN REVIEW for a multi-family residential development in conjunction with an existing golf course on a 1.7 acre portion of 8.05 acres in a C-2 (General Commercial District) Zone within the Southern Highlands Planned Community (PCO) Overlay.  Generally located north of Robert Trent Jones Lane and west of Southern Highlands Parkway within Enterprise.  JJ/bb/kh  (For possible action)</t>
-  </si>
-  <si>
-    <t>Clark County | 163 At Casino Drive casino: Approve and authorize the Chair to sign Supplemental No. 8 to the interlocal contract between Clark County and Regional Flood Control District to extend the contract term for design of the State Route 163 at Casino Drive project.  (For possible action)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | Visible Noise family entertainment centre: UC-26-0303-VISIBLE NOISE, LLC:
-HOLDOVER USE PERMIT for a proposed recreational or entertainment facility within an existing office/warehouse complex on a portion of 5.31 acres in an IP (Industrial Park) Zone within the Airport Environs (AE-60) Overlay. Generally located west of Tenaya Way and north of Sunset Road within Spring Valley.  MN/rp/cv  (For possible action)</t>
-  </si>
-  <si>
-    <t>Clark County | Hilton Resorts resort: 3. UC-26-0373-HILTON RESORTS CORPORATION: USE PERMIT for a monorail on approximately 21 acres in an RM50 (Residential Multi-Family 50) Zone, a CR (Commercial Resort) Zone, and an IL (Industrial Light)</t>
+    <t>Phoenix | Rezoning Application Z-15-26-2 - Southwest Corner of 56th Street and Ranger: Public Hearing and Ordinance Adoption - Rezoning Application Z-15-26-2 - Southwest Corner of 56th Street and Ranger Drive (Ordinance G-7525) - District 2</t>
+  </si>
+  <si>
+    <t>2026-06-30 | Phoenix</t>
+  </si>
+  <si>
+    <t>https://phoenix.legistar.com/gateway.aspx?M=l&amp;ID=35401</t>
+  </si>
+  <si>
+    <t>Phoenix | North Phoenix Growers, LLC et. al leisure development: Amend City Code - Ordinance Adoption - Rezoning Application Z-25-26-1-2 - Approximately 430 Feet South of the Southeast Corner of 19th Avenue and Jomax Road (Ordinance G-7529) - Districts 1 &amp; 2</t>
+  </si>
+  <si>
+    <t>https://phoenix.legistar.com/gateway.aspx?M=l&amp;ID=35400</t>
+  </si>
+  <si>
+    <t>Phoenix | Children's Museum of Phoenix: Children's Museum of Phoenix</t>
+  </si>
+  <si>
+    <t>https://phoenix.legistar.com/gateway.aspx?M=l&amp;ID=35482</t>
+  </si>
+  <si>
+    <t>Phoenix | Woodland Plaza, LLC, et.al leisure development: Amend City Code - Ordinance Adoption - Rezoning Application Z-145-24-1 - Approximately 200 Feet North of the Northwest Corner of 35th Avenue and Bell Road (Ordinance G-7528) - District 1</t>
+  </si>
+  <si>
+    <t>https://phoenix.legistar.com/gateway.aspx?M=l&amp;ID=35398</t>
+  </si>
+  <si>
+    <t>Phoenix | Randy Raskin, 43rd Ave leisure development: Amend City Code - Ordinance Adoption - Rezoning Application PHO-1-26--Z-29-23-7(8) - Approximately 300 Feet East of the Northeast Corner of 43rd Avenue and Baseline Road (Ordinance G-7531) - District 8</t>
+  </si>
+  <si>
+    <t>https://phoenix.legistar.com/gateway.aspx?M=l&amp;ID=35415</t>
+  </si>
+  <si>
+    <t>Phoenix | Larry Miller, Matrix at Dobbins leisure development: Amend City Code - Ordinance Adoption - Rezoning Application PHO-1-26--Z-45-22-8 - Southeast Corner of 59th Avenue and Dobbins Road (Ordinance G-7532) - District 8</t>
+  </si>
+  <si>
+    <t>https://phoenix.legistar.com/gateway.aspx?M=l&amp;ID=35416</t>
+  </si>
+  <si>
+    <t>Phoenix | VTHQ leisure development: Amend City Code - Ordinance Adoption - Rezoning Application Z-27-26-8 - Southwest Corner of 14th Street and Hess Avenue (Ordinance G-7530) - District 8</t>
+  </si>
+  <si>
+    <t>https://phoenix.legistar.com/gateway.aspx?M=l&amp;ID=35403</t>
+  </si>
+  <si>
+    <t>Phoenix | Liquor License - Fire N Ice Arena - District 2: Liquor License - Fire N Ice Arena - District 2</t>
+  </si>
+  <si>
+    <t>2026-06-16 | Phoenix</t>
+  </si>
+  <si>
+    <t>https://phoenix.legistar.com/Legislation.aspx#matter-35274</t>
+  </si>
+  <si>
+    <t>Phoenix | Laveen Baseline leisure development: Amend Ordinance S-47581 and Development Agreement (City Contract 157059) with Laveen Baseline LLC (Ordinance S-53031) - Districts 7 &amp; 8</t>
+  </si>
+  <si>
+    <t>https://phoenix.legistar.com/Legislation.aspx#matter-35236</t>
+  </si>
+  <si>
+    <t>Phoenix | ADD-ON - Tohono O'odham Nation Tribal 2025 Gaming Grants (Ordinance S-52900): ADD-ON - Tohono O'odham Nation Tribal 2025 Gaming Grants (Ordinance S-52900) - Citywide</t>
+  </si>
+  <si>
+    <t>2026-05-19 | Phoenix</t>
+  </si>
+  <si>
+    <t>https://phoenix.legistar.com/gateway.aspx?M=l&amp;ID=35247</t>
+  </si>
+  <si>
+    <t>Clark County | Club 36 Master Association integrated resort: 4. UC-26-0383-BG CLUB 36 MASTER ASSOCIATION: USE PERMIT for a monorail on approximately 80 acres in a CR (Commercial Resort) Zone and a CG (Commercial General) Zone within the Airport Environs (AE-60,</t>
   </si>
   <si>
     <t>2026-07-28 | Clark County</t>
   </si>
   <si>
-    <t>https://www.clarkcountynv.gov/adobe/assets/urn:aaid:aem:7592f7a2-1607-4db1-84fd-1e20f3737ec6/original/as/Winchester-Agenda-072826.pdf#item-uc-26-0373</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | Buona Vita resort: 2. AR-26-400068 (ET-25-400074(UC-23-0659))-BUONA VITA, LLC: USE PERMIT FIRST APPLICATION FOR REVIEW for daycare and school. WAIVERS OF DEVELOPMENT STANDARDS for the following: 1) trash enclosure; and </t>
-  </si>
-  <si>
-    <t>https://www.clarkcountynv.gov/adobe/assets/urn:aaid:aem:7592f7a2-1607-4db1-84fd-1e20f3737ec6/original/as/Winchester-Agenda-072826.pdf#item-ar-26-400068+et-25-400074+uc-23-0659</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | Tropicana Land resort: WS-26-0113-TROPICANA LAND, LLC:
-HOLDOVER WAIVER OF DEVELOPMENT STANDARDS for modified driveway geometrics.
-DESIGN REVIEW for a resort hotel on a 26.11 acre portion of 35.11 acres in a CR (Commercial Resort) Zone within the Airport Environs (AE-60) Overlay. Generally located south of Tropicana Avenue and east of Las Vegas Boulevard South within Paradise.  JG/nm/kh  (For possible action)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | South Decatur Holding CO leisure development: PA-26-700010-SOUTH DECATUR HOLDING CO., LLC:
-PLAN AMENDMENT to redesignate the existing land use category from Neighborhood Commercial (NC) to Compact Neighborhood (CN) on 2.64 acres.  Generally located east of Decatur Boulevard and south of Moberly Avenue (alignment) within Enterprise. MN/rk (For possible action)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | Church Searchlight Community leisure development: PA-26-700019-CHURCH SEARCHLIGHT COMMUNITY:
-PLAN AMENDMENT to redesignate the existing land use category from Public Use (PU) to Neighborhood commercial (NC) on 4.8 acres.   Generally located west of US Highway 95 and north of State Route 164 within Searchlight. MN/rk  (For possible action)</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110428</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | G D Carden Entertainment museum: ET-26-400054 (UC-25-0072)-GD CARDEN ENTERTAINMENT, LLC:
-USE PERMITS FIRST EXTENSION OF TIME for the following: 1) recreational or entertainment facility; 2) museum; and 3) live entertainment. 
-WAIVERS OF DEVELOPMENT STANDARDS for the following: 1) eliminate and reduce setbacks; 2) reduce parking requirements; 3) waive full off-site improvements; 4) reduce driveway approach distance; 5) reduce driveway departure distance; and 6) reduce driveway width.
-DESIGN REVIEW for a recreational or entertainment facility and museum on 1.82 acres in an RS20 (Residential Single-Family 20) Zone within a Historic Designation (HDO) Overlay.  Generally located north of Vegas Drive and west of Valley Drive within the Lone Mountain Planning Area.  WM/rr/cv  (For possible action)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | Beltway 101, LLC &amp; Blue 10 leisure development: PA-26-700025-BELTWAY 101, LLC &amp; BLUE 10, LLC:
-PLAN AMENDMENT to redesignate the existing land use category from Neighborhood Commercial (NC) to Compact Neighborhood (CN) on 4.51 acres. Generally located north of Blue Diamond Road and west of Montessouri Street (alignment) within Enterprise. JJ/gc (For possible action)</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110451</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | Shamaim Henderson family entertainment centre: UC-26-0309-SHAMAIM HENDERSON, LLC:
-USE PERMITS for the following: 1) an avocational or vocational training facility; and 2) a recreational or entertainment facility on a portion of 5.11 acres in an IL (Industrial Light) Zone and an IP (Industrial Park) Zone within the Airport Environs (AE-60 &amp; AE-65) Overlay. Generally located south of Pilot Road and west of Bermuda Road within Enterprise.  MN/hw/cv  (For possible action)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | BOLOGNESE, JOSEPH &amp; VIVI A: PLAN AMENDMENT to redesignate the existing land use: PA-26-700026-BOLOGNESE, JOSEPH &amp; VIVI A:
-PLAN AMENDMENT to redesignate the existing land use category from Corridor Mixed-Use (CM) to Compact Neighborhood (CN) on 1.93 acres.  Generally located north of Serene Avenue and east of Grand Canyon Drive within Enterprise. JJ/rk (For possible action)</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/Legislation.aspx#matter-110398</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | Diamond Quail leisure development: PA-26-700018-DIAMOND QUAIL, LLC:
-PLAN AMENDMENT to redesignate the existing land use category from Neighborhood Commercial (NC) to Business Employment (BE) on 1.24 acres.   Generally located north of Quail Avenue and east of Santa Margarita Street (alignment) within Spring Valley. MN/gc (For possible action)</t>
+    <t>https://www.clarkcountynv.gov/adobe/assets/urn:aaid:aem:7592f7a2-1607-4db1-84fd-1e20f3737ec6/original/as/Winchester-Agenda-072826.pdf#item-uc-26-0383</t>
+  </si>
+  <si>
+    <t>Clark County | Heart Hotel / Kulik River: Las Vegas Topic Kulik River Capital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clark County | Mirage Propco casino: DR-26-0313-MIRAGE PROPCO, LLC:
+DESIGN REVIEW for a proposed theater expansion in conjunction with a previously approved resort hotel (Hard Rock Hotel &amp; Casino) on a portion of 76.93 acres in a CR (Commercial Resort) Zone. Generally located west of Las Vegas Boulevard South and south of Spring Mountain Road within Paradise.  TS/hw/cv  (For possible action)</t>
+  </si>
+  <si>
+    <t>Clark County | Toll South LV leisure development: ORD-26-900159: Conduct a public hearing on an ordinance to consider adoption of a Development Agreement with Toll South LV LLC for a single-family residential subdivision on 0.89 acres, generally located east of Hinson Street and north of Silverado Ranch Boulevard within Enterprise. JJ/tpd (For possible action)</t>
+  </si>
+  <si>
+    <t>Clark County | BDA South leisure development: ORD-26-900280: Conduct a public hearing on an ordinance to consider adoption of a Development Agreement with BDA South, LLC for a vehicle wash on 1.08 acres, generally located north of Wigwam Avenue and east of Arville Street within Enterprise. JJ/tpd (For possible action)</t>
+  </si>
+  <si>
+    <t>Clark County | World Buddhism Association Headquarters &amp; MGM-Grand Bally's integrated resort: 4. AR-26-400041 (UC-25-0544)-WORLD BUDDHISM ASSOCIATION HEADQUARTERS &amp; MGM-GRAND BALLY'S, LLC LEASE: USE PERMIT FIRST APPLICATION FOR REVIEW for a recreational or entertainment facility. DESIGN REVIEW</t>
+  </si>
+  <si>
+    <t>Clark County | ZL II leisure development: ORD-26-900259: Conduct a public hearing on an ordinance to consider adoption of a Development Agreement with ZL II, LLC for an avocational or vocational training facility and parking lot expansion on 12.04 acres, generally located east of El Camino Road and north of Rafael Rivera Way within Enterprise. MN/jl (For possible action)</t>
   </si>
   <si>
     <t>2026-07-07 | Clark County</t>
   </si>
   <si>
-    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110321</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | RDXNWP family entertainment centre: UC-26-0302-RDXNWP, LLC:
-USE PERMIT to allow outdoor storage. 
-WAIVERS OF DEVELOPMENT STANDARDS for the following: 1) eliminate electric vehicle charging spaces; and 2) modified driveway geometrics.
-DESIGN REVIEW for a proposed recreational and entertainment facility (ice rink) within an existing shopping center on a 7.02 acre portion of 10.85 acres in a CG (Commercial General) Zone within the Airport Environs (AE-60) Overlay. Generally located south of Russell Road and west of Decatur Boulevard within Spring Valley.  MN/bb/kh  (For possible action)</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110314</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | Sustainable Development Fund 1 leisure development: PA-26-700021-SUSTAINABLE DEVELOPMENT FUND 1, LLC:
-HOLDOVER PLAN AMENDMENT to redesignate the existing land use category from Neighborhood Commercial (NC) to Business Employment (BE) on 0.95 acres.  Generally located east of Decatur Boulevard and north of Eldorado Lane within Enterprise. MN/rk  (For possible action)</t>
-  </si>
-  <si>
-    <t>2026-07-06 | Clark County</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110272</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | CITY OF LAS VEGAS: HOLDOVER PLAN AMENDMENT to redesignate the existing land use: PA-26-700022-CITY OF LAS VEGAS:
-HOLDOVER PLAN AMENDMENT to redesignate the existing land use category from Public Use (PU) to Urban Neighborhood (UN) on a 15.20 acre portion of a 31.58 acre site. Generally located south of Vegas Valley Drive and west of Tree Line Drive (alignment) within Sunrise Manor. TS/gc (For possible action)</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110275</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | Buffalo Amigos, LLC Etal &amp; Silver Serene leisure development: PA-26-700004-BUFFALO AMIGOS, LLC ETAL &amp; SILVER SERENE, LLC:
-AMENDED HOLDOVER PLAN AMENDMENT to redesignate the existing land use category from Ranch Estate Neighborhood (RN) to Low-Intensity Suburban Neighborhood (LN) on 5.10 acres (previously notified as 5.0 acres). Generally located west of Buffalo Drive and north of Torino Avenue within Enterprise.  JJ/rk (For possible action)</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110255</t>
-  </si>
-  <si>
-    <t>Clark County | 215 And Windmill Lane leisure development: Approve and authorize the Community Housing Administrator to nominate a 20-acre site known as APN# 177-11-401-004, a Bureau of Land Management (BLM) site reserved by the County for affordable housing located at the northeast corner of I-215 and Windmill Lane, for use as affordable housing pursuant to Section 7(b) of the Southern Nevada Public Lands Management Act; approve and authorize the Director of Real Property Management to accept conveyance of the site from the BLM, and subsequently transfer the site via quitclaim deed and disposition and development agreement to Coordinated Living of Southern Nevada for the development of affordable housing; and authorize the Director of Real Property Management, or her designee, to sign any documents related thereto (For possible action.)</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110284</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clark County | Horizon West Homes leisure development: PA-26-700017-HORIZON WEST HOMES, LLC:
-HOLDOVER PLAN AMENDMENT to redesignate the land use category from Mid-Intensity Suburban Neighborhood (MN) to Compact Neighborhood (CN) on 1.44 acres.  Generally located east of Hualapai Way and north of Serene Avenue within Enterprise.  JJ/rk  (For possible action)</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110264</t>
-  </si>
-  <si>
-    <t>Clark County | REFRIGERATION SUPPLIES DISTRIBUTOR: DESIGN REVIEW for a proposed: 6. DR-26-0236-REFRIGERATION SUPPLIES DISTRIBUTOR: DESIGN REVIEW for a proposed office/warehouse building on 1.91 acres in an IL (Industrial Light) Zone within the Airport Environs (AE-60) Overlay. Gen</t>
-  </si>
-  <si>
-    <t>2026-05-12 | Clark County</t>
-  </si>
-  <si>
-    <t>https://www.clarkcountynv.gov/adobe/assets/urn:aaid:aem:d8194047-38e8-4588-b3c6-cfb5682e7f84/original/as/Paradise-Minutes-051226.pdf#item-dr-26-0236</t>
-  </si>
-  <si>
-    <t>Clark County | LV Diamond Property I resort: 6. AR-26-400027 (UC-22-0556)-LV DIAMOND PROPERTY I, LLC: WAIVER OF DEVELOPMENT STANDARDS SECOND APPLICATION FOR REVIEW to eliminate street landscaping for an existing racetrack, recreational facility,</t>
-  </si>
-  <si>
-    <t>2026-04-28 | Clark County</t>
-  </si>
-  <si>
-    <t>https://www.clarkcountynv.gov/adobe/assets/urn:aaid:aem:f1a4b305-a7fb-49f7-a5fe-06ab39312955/original/as/Paradise-Minutes-042826.pdf#item-ar-26-400027+uc-22-0556</t>
-  </si>
-  <si>
-    <t>Clark County | MGM Resorts Festival Grounds museum: 8. VS-26-0213-MGM RESORTS FESTIVAL GROUNDS, LLC: VACATE AND ABANDON easements of interest to Clark County located between Reno Avenue and Mandalay Bay Road, and Giles Street and Las Vegas Boulevard So</t>
-  </si>
-  <si>
-    <t>https://www.clarkcountynv.gov/adobe/assets/urn:aaid:aem:f1a4b305-a7fb-49f7-a5fe-06ab39312955/original/as/Paradise-Minutes-042826.pdf#item-vs-26-0213</t>
-  </si>
-  <si>
-    <t>Las Vegas | Top Gun Las Vegas: Top Gun Vegas Locks South Strip Site at 4815 Las Vegas ...</t>
-  </si>
-  <si>
-    <t>Las Vegas | Plaza Hotel &amp; Casino casino: 14. For possible action to approve the ratification of the Commission for the Las Vegas Centennial funding allocation to be used for the planning and running of the 2027, 2028, and 2029 Las Vegas Days</t>
-  </si>
-  <si>
-    <t>2026-07-01 | Las Vegas</t>
-  </si>
-  <si>
-    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=42864#item-h34a32883beda</t>
-  </si>
-  <si>
-    <t>Las Vegas | possible action to approve the ratification of the Commission for the Las Vegas: 11. For possible action to approve the ratification of the Commission for the Las Vegas Centennial award of $160,000 to the Neon Museum for the costs associated with the planning and running of a four</t>
-  </si>
-  <si>
-    <t>2026-06-03 | Las Vegas</t>
-  </si>
-  <si>
-    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=42406#item-h437a333ac173</t>
-  </si>
-  <si>
-    <t>Las Vegas | multifamily and mixed-use development that includes a residential component as: 40. Bill No. 2026-16 - For possible action - Authorizes multifamily and mixed-use development that includes a residential component as a conditional use on property zoned for commercial use, in accord</t>
-  </si>
-  <si>
-    <t>Las Vegas | various provisions of LVMC Title 19 to establish the Transit Oriented: 36. Bill No. 2026-13 - For possible action - Amends various provisions of LVMC Title 19 to establish the Transit Oriented Development Overlay District and make parallel adjustments. Sponsored by: Coun</t>
-  </si>
-  <si>
-    <t>2026-05-06 | Las Vegas</t>
-  </si>
-  <si>
-    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=42376#item-ha8f0435b0451</t>
-  </si>
-  <si>
-    <t>Las Vegas | Brandywine Bookmaking casino: 18. For possible action to approve a new Non Restricted Gaming license for BRANDYWINE BOOKMAKING LLC dba WILLIAM HILL RACE &amp; SPORTS BOOK dba PLAZA HOTEL &amp; CASINO at 1 South Main Street - Ward 5 (Summe</t>
-  </si>
-  <si>
-    <t>2026-04-15 | Las Vegas</t>
-  </si>
-  <si>
-    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=42356#item-h2667b1bb6acb</t>
-  </si>
-  <si>
-    <t>Las Vegas | 2000 South Las Vegas Boulevard casino: 14. For possible action to approve a new Non Restricted Gaming license for WILLIAM HILL l dba WILLIAM HILL RACE &amp; SPORTS BOOK db at THE STRAT, HOTEL, CASINO &amp; TOWER at 2000 South Las Vegas Boulevard -</t>
-  </si>
-  <si>
-    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=42356#item-h836f352fe1c5</t>
-  </si>
-  <si>
-    <t>Las Vegas | WILLIAM HILL ll casino: 15. For possible action to approve a new Non Restricted Gaming license for WILLIAM HILL ll dba WILLIAM HILL RACE &amp; SPORTS BOOK dba FOUR QUEENS HOTEL AND CASINO at 202 Fremont Street - Ward 3 (Diaz) Ag</t>
-  </si>
-  <si>
-    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=42356#item-ha1a186745a91</t>
-  </si>
-  <si>
-    <t>Las Vegas | 221 North Rampart Boulevard casino: 19. For possible action to approve a new Non Restricted Gaming license for WILLIAM HILL1 dba CAESARS SPORTSBOOK db at THE RESORT AT SUMMERLIN at 221 North Rampart Boulevard - Ward 2 (Kelley) Agenda Su</t>
-  </si>
-  <si>
-    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=42356#item-h2fea74770792</t>
-  </si>
-  <si>
-    <t>Las Vegas | Fifth Street Gaming casino: 10. For possible action to approve a One-Day Opening for a Non-Restricted Gaming license for FIFTH STREET GAMING LLC dba FIFTH STREET GAMING LLC db at WESTERN HOTEL &amp; CASINO at 899 Fremont Street - Wa</t>
-  </si>
-  <si>
-    <t>2026-03-18 | Las Vegas</t>
-  </si>
-  <si>
-    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=42326#item-h28eb1d558fc2</t>
-  </si>
-  <si>
-    <t>Las Vegas | 000 For The Maryland Parkway leisure development: 25. For possible action to approve Supplemental No. 6 to Interlocal Contract 1164 between the Cities of Las Vegas (CLV), North Las Vegas, Henderson, Boulder City and Mesquite, Clark County, and the Re</t>
-  </si>
-  <si>
-    <t>2026-01-21 | Las Vegas</t>
-  </si>
-  <si>
-    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=42256#item-hfcc9035cbd00</t>
-  </si>
-  <si>
-    <t>Las Vegas | Proview Series 39 casino: 15. For possible action to approve a Parking Lease Agreement between Proview Series 39, LLC, and the City of Las Vegas (City) where the City will manage and operate a fifty-nine (59) space parking lot</t>
-  </si>
-  <si>
-    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=42256#item-h70b1f823b194</t>
-  </si>
-  <si>
-    <t>Las Vegas | KLA Capital Series 7 casino: 16. For possible action to approve a Parking Lease Agreement between KLA Capital Series 7, LLC, and the City of Las Vegas (City) where the City will manage and operate a nineteen (19) space parking lo</t>
-  </si>
-  <si>
-    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=42256#item-he8c543b347e4</t>
-  </si>
-  <si>
-    <t>Las Vegas | Nevada Test Site Historical Foundation museum: 11. For possible action to approve the ratification of the Commission for the Las Vegas Centennial funding allocation for the creation and installation of a permanent educational museum exhibit and to</t>
-  </si>
-  <si>
-    <t>2026-01-07 | Las Vegas</t>
-  </si>
-  <si>
-    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=42246#item-h2e63d4603e2f</t>
-  </si>
-  <si>
-    <t>Las Vegas | 2427 South Las Vegas Boulevard casino: 12. For possible action to approve a One-Day Opening for a Non-Restricted Gaming License for UNITED COIN MACHINE dba CENTURY GAMING TECHNOLOGIES db at HOLY COW! CASINO CAFE at 2427 South Las Vegas Bou</t>
-  </si>
-  <si>
-    <t>2025-12-17 | Las Vegas</t>
-  </si>
-  <si>
-    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=42132#item-h9540a7706bbe</t>
-  </si>
-  <si>
-    <t>Las Vegas | possible action to approve the Third Amendment to Lease and Operating Agreement: 18. For possible action to approve the Third Amendment to Lease and Operating Agreement between The Smith Center for Performing Arts and the City of Las Vegas (City) where the parking facility informa</t>
+    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110310</t>
+  </si>
+  <si>
+    <t>Clark County | Cimarron Spring Deux LLC, A &amp; A Revocable Living Trust leisure development: ORD-26-900221: Conduct a public hearing on an ordinance to consider adoption of a Development Agreement with Cimarron Spring Deux LLC, A &amp; A Revocable Living Trust, and A &amp; A III LLC for a single-family development on 2.54 acres, generally located west of Hinson Street and south of Richmar Avenue within Enterprise. JJ/tpd (For possible action)</t>
+  </si>
+  <si>
+    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110308</t>
+  </si>
+  <si>
+    <t>Clark County | Ruby Holdings museum: 5. UC-26-0156-RUBY HOLDINGS, LLC: USE PERMITS for the following: 1) museum; and 2) office as a primary use. WAIVER OF DEVELOPMENT STANDARDS to reduce parking. DESIGN REVIEW for a proposed museum in co</t>
+  </si>
+  <si>
+    <t>2026-04-14 | Clark County</t>
+  </si>
+  <si>
+    <t>https://www.clarkcountynv.gov/adobe/assets/urn:aaid:aem:13a91c3e-05d2-48c5-bc38-a8b251f9bf46/original/as/Paradise-Minutes-041426.pdf#item-uc-26-0156</t>
+  </si>
+  <si>
+    <t>Nashville | 12802 Old Hickory Boulevard mixed-use development: An ordinance to amend Title 17 of the Metropolitan Code of Laws, the Zoning Ordinance of The Metropolitan Government of Nashville and Davidson County, by changing from AR2a to SP zoning for property located at 12802 Old Hickory Boulevard, approximately 148 feet southwest of Logistics Way (3.6 acres), to permit a mixed use development, all of which is described herein (Proposal No. 2026SP-025-001).</t>
+  </si>
+  <si>
+    <t>Nashville | amending Chapter 17.08 of the Metropolitan Code of Laws to modify the Zoning: An ordinance amending Chapter 17.08 of the Metropolitan Code of Laws to modify the Zoning District Land Use Table to reflect recent amendments to the Zoning Code (Proposal No. 2026Z-014-TX-001).</t>
+  </si>
+  <si>
+    <t>https://nashville.legistar.com/gateway.aspx?M=l&amp;ID=20861</t>
+  </si>
+  <si>
+    <t>Nashville | approving Amendment No. 6 to the Arts Center Redevelopment Plan, Amendment No. 1: An ordinance approving Amendment No. 6 to the Arts Center Redevelopment Plan, Amendment No. 1 to the Bordeaux Redevelopment Plan, Amendment No. 1 to the Central State Redevelopment Plan, Amendment No. 6 to the Phillips-Jackson Redevelopment Plan, Amendment No. 9 to the Rutledge Hill Redevelopment Plan, and Amendment No. 1 to the Skyline Redevelopment Plan. (Proposal No. 2026M-002OT-001)</t>
+  </si>
+  <si>
+    <t>https://nashville.legistar.com/gateway.aspx?M=l&amp;ID=20850</t>
+  </si>
+  <si>
+    <t>Nashville | to authorize building material restrictions and requirements for BL2026-1474: An ordinance to amend Title 17 of the Metropolitan Code of Laws, the Zoning Ordinance of The Metropolitan Government of Nashville and Davidson County, by changing from IR to SP zoning for property located at 1205 2nd Avenue North, approximately 129 feet north of Madison Street (0.46 acres), to permit a mixed use development, all of which is described herein (Proposal No. 2026SP-024-001).</t>
+  </si>
+  <si>
+    <t>Central Florida Tourism Oversight District | 10450 Turkey Lake Road leisure development: Contract between CFTOD and Tower Engineering Inc. approved by the Board at the November 21, 2025, meeting</t>
+  </si>
+  <si>
+    <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/1-23-2026-BOS-Agenda-Packet-FINALcs.pdf#item-9.1-p276</t>
+  </si>
+  <si>
+    <t>Central Florida Tourism Oversight District | CFTOD / Walt Disney World: Approve the District Administrator to execute a Non-exclusive temporary easement with permanent easement to Walt Disney Parks &amp; Resorts, U.S. Inc for underground communication lines</t>
+  </si>
+  <si>
+    <t>Anaheim | OCVibe: 4. Determinar sobre la base de la evidencia presentada por Anaheim Real Estate Partners, LLC, TS Anaheim, LLC y FCD, LLC (OCVIBE), que el propietario de la propiedad ha cumplido de buena fe con los té</t>
+  </si>
+  <si>
+    <t>Las Vegas | 500 North Casino Center Drive casino: 24. For possible action to approve award of Contract No. 260025-JG, Prime Design Services for Fire Administration Restrooms/Central Plant Modernization, located at 500 North Casino Center Drive - Depa</t>
   </si>
   <si>
     <t>2025-10-15 | Las Vegas</t>
   </si>
   <si>
-    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=41822#item-h511ab179299a</t>
+    <t>https://lasvegas.primegov.com/Portal/Meeting?meetingTemplateId=41822#item-hb68c01f5db23</t>
+  </si>
+  <si>
+    <t>Bonita Springs | 8910 Terrene Ct leisure development: Bonita Bay Lake 21 Restoration (250609-53694_36-114553-P)</t>
+  </si>
+  <si>
+    <t>2025-10-14 | Bonita Springs</t>
+  </si>
+  <si>
+    <t>https://www.sfwmd.gov/regpermitting#erp-250609-53694_36-114553-P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Antonio | Weston Urban leisure development: Discussion and possible action to authorize execution of a Master Economic Incentive Agreement between Weston Urban, LLC and the City of San Antonio as a source of funding for public improvements related to the redevelopment of the property located at 322 W. Commerce, for an amount up to $250,000.
+</t>
   </si>
   <si>
     <t>Coverage note</t>
   </si>
   <si>
-    <t>Coverage is limited to Clark County, Las Vegas. Projects outside it exist in our register and are not reported here.</t>
+    <t>Coverage is limited to Altamonte Springs, Anaheim, Atlanta, Bonita Springs, Central Florida Tourism Oversight District, Clark County, Kissimmee, Lake Buena Vista, Las Vegas, Miami-Dade County, Nashville, Oakland, Phoenix, San Antonio, South Florida, Walt Disney World. Projects outside it exist in our register and are not reported here.</t>
   </si>
   <si>
     <t>The period is July 2026. Activity outside it is not included even where it concerns the same project.</t>
@@ -832,7 +725,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -925,919 +818,732 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C11" t="s">
         <v>21</v>
       </c>
       <c r="D11" t="s">
+        <v>18</v>
+      </c>
+      <c r="E11" t="s">
         <v>22</v>
-      </c>
-      <c r="E11" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
         <v>24</v>
       </c>
       <c r="D12" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="E12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
         <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s">
         <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E14" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D15" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E15" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B16" t="s">
         <v>16</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D16" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E16" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B17" t="s">
         <v>16</v>
       </c>
       <c r="C17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" t="s">
         <v>37</v>
       </c>
-      <c r="D17" t="s">
-        <v>30</v>
-      </c>
       <c r="E17" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B18" t="s">
         <v>16</v>
       </c>
       <c r="C18" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D18" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="E18" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B19" t="s">
         <v>16</v>
       </c>
       <c r="C19" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D19" t="s">
         <v>42</v>
       </c>
       <c r="E19" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="B20" t="s">
         <v>16</v>
       </c>
       <c r="C20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D20" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="E20" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B21" t="s">
         <v>16</v>
       </c>
       <c r="C21" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D21" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="E21" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B22" t="s">
         <v>16</v>
       </c>
       <c r="C22" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D22" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="E22" t="s">
-        <v>19</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B23" t="s">
         <v>16</v>
       </c>
       <c r="C23" t="s">
+        <v>54</v>
+      </c>
+      <c r="D23" t="s">
         <v>50</v>
       </c>
-      <c r="D23" t="s">
-        <v>18</v>
-      </c>
       <c r="E23" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B24" t="s">
         <v>16</v>
       </c>
       <c r="C24" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D24" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="E24" t="s">
-        <v>36</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B25" t="s">
         <v>16</v>
       </c>
       <c r="C25" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D25" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="E25" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B26" t="s">
         <v>16</v>
       </c>
       <c r="C26" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="D26" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E26" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B27" t="s">
         <v>16</v>
       </c>
       <c r="C27" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D27" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E27" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B28" t="s">
         <v>16</v>
       </c>
       <c r="C28" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D28" t="s">
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="E28" t="s">
-        <v>31</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B29" t="s">
         <v>16</v>
       </c>
       <c r="C29" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="D29" t="s">
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="E29" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B30" t="s">
         <v>16</v>
       </c>
       <c r="C30" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D30" t="s">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="E30" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B31" t="s">
         <v>16</v>
       </c>
       <c r="C31" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="D31" t="s">
-        <v>30</v>
+        <v>73</v>
       </c>
       <c r="E31" t="s">
-        <v>40</v>
+        <v>74</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B32" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C32" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="D32" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E32" t="s">
-        <v>64</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B33" t="s">
         <v>16</v>
       </c>
       <c r="C33" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="D33" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="E33" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B34" t="s">
         <v>16</v>
       </c>
       <c r="C34" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="D34" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="E34" t="s">
-        <v>67</v>
+        <v>38</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B35" t="s">
         <v>16</v>
       </c>
       <c r="C35" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="D35" t="s">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="E35" t="s">
-        <v>70</v>
+        <v>40</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B36" t="s">
         <v>16</v>
       </c>
       <c r="C36" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="D36" t="s">
-        <v>69</v>
+        <v>34</v>
       </c>
       <c r="E36" t="s">
-        <v>72</v>
+        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B37" t="s">
         <v>16</v>
       </c>
       <c r="C37" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="D37" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="E37" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B38" t="s">
         <v>16</v>
       </c>
       <c r="C38" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="D38" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="E38" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B39" t="s">
         <v>16</v>
       </c>
       <c r="C39" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="D39" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="E39" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B40" t="s">
         <v>16</v>
       </c>
       <c r="C40" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="D40" t="s">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="E40" t="s">
-        <v>81</v>
+        <v>43</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B41" t="s">
         <v>16</v>
       </c>
       <c r="C41" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="D41" t="s">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="E41" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B42" t="s">
         <v>16</v>
       </c>
       <c r="C42" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D42" t="s">
-        <v>85</v>
+        <v>42</v>
       </c>
       <c r="E42" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B43" t="s">
         <v>16</v>
       </c>
       <c r="C43" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="D43" t="s">
-        <v>88</v>
+        <v>42</v>
       </c>
       <c r="E43" t="s">
-        <v>89</v>
+        <v>45</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B44" t="s">
         <v>16</v>
       </c>
       <c r="C44" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D44" t="s">
-        <v>88</v>
+        <v>28</v>
       </c>
       <c r="E44" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B45" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C45" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D45" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="E45" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B46" t="s">
         <v>16</v>
       </c>
       <c r="C46" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D46" t="s">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="E46" t="s">
-        <v>95</v>
+        <v>22</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B47" t="s">
         <v>16</v>
       </c>
       <c r="C47" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E47" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B48" t="s">
         <v>16</v>
       </c>
       <c r="C48" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D48" t="s">
-        <v>33</v>
+        <v>102</v>
       </c>
       <c r="E48" t="s">
-        <v>34</v>
+        <v>103</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B49" t="s">
         <v>16</v>
       </c>
       <c r="C49" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D49" t="s">
-        <v>101</v>
+        <v>31</v>
       </c>
       <c r="E49" t="s">
-        <v>102</v>
+        <v>32</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>44</v>
+        <v>105</v>
       </c>
       <c r="B50" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C50" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D50" t="s">
-        <v>104</v>
+        <v>14</v>
       </c>
       <c r="E50" t="s">
-        <v>105</v>
+        <v>14</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>44</v>
+        <v>105</v>
       </c>
       <c r="B51" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C51" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D51" t="s">
-        <v>104</v>
+        <v>14</v>
       </c>
       <c r="E51" t="s">
-        <v>107</v>
+        <v>14</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>44</v>
+        <v>105</v>
       </c>
       <c r="B52" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C52" t="s">
         <v>108</v>
       </c>
       <c r="D52" t="s">
-        <v>104</v>
+        <v>14</v>
       </c>
       <c r="E52" t="s">
-        <v>109</v>
+        <v>14</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>44</v>
+        <v>105</v>
       </c>
       <c r="B53" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C53" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D53" t="s">
-        <v>104</v>
+        <v>14</v>
       </c>
       <c r="E53" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>44</v>
-      </c>
-      <c r="B54" t="s">
-        <v>16</v>
-      </c>
-      <c r="C54" t="s">
-        <v>112</v>
-      </c>
-      <c r="D54" t="s">
-        <v>113</v>
-      </c>
-      <c r="E54" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>44</v>
-      </c>
-      <c r="B55" t="s">
-        <v>16</v>
-      </c>
-      <c r="C55" t="s">
-        <v>115</v>
-      </c>
-      <c r="D55" t="s">
-        <v>116</v>
-      </c>
-      <c r="E55" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>44</v>
-      </c>
-      <c r="B56" t="s">
-        <v>16</v>
-      </c>
-      <c r="C56" t="s">
-        <v>118</v>
-      </c>
-      <c r="D56" t="s">
-        <v>116</v>
-      </c>
-      <c r="E56" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>44</v>
-      </c>
-      <c r="B57" t="s">
-        <v>16</v>
-      </c>
-      <c r="C57" t="s">
-        <v>120</v>
-      </c>
-      <c r="D57" t="s">
-        <v>116</v>
-      </c>
-      <c r="E57" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>44</v>
-      </c>
-      <c r="B58" t="s">
-        <v>16</v>
-      </c>
-      <c r="C58" t="s">
-        <v>122</v>
-      </c>
-      <c r="D58" t="s">
-        <v>123</v>
-      </c>
-      <c r="E58" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>44</v>
-      </c>
-      <c r="B59" t="s">
-        <v>16</v>
-      </c>
-      <c r="C59" t="s">
-        <v>125</v>
-      </c>
-      <c r="D59" t="s">
-        <v>126</v>
-      </c>
-      <c r="E59" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>44</v>
-      </c>
-      <c r="B60" t="s">
-        <v>16</v>
-      </c>
-      <c r="C60" t="s">
-        <v>128</v>
-      </c>
-      <c r="D60" t="s">
-        <v>129</v>
-      </c>
-      <c r="E60" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>131</v>
-      </c>
-      <c r="B61" t="s">
-        <v>12</v>
-      </c>
-      <c r="C61" t="s">
-        <v>132</v>
-      </c>
-      <c r="D61" t="s">
-        <v>14</v>
-      </c>
-      <c r="E61" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>131</v>
-      </c>
-      <c r="B62" t="s">
-        <v>12</v>
-      </c>
-      <c r="C62" t="s">
-        <v>133</v>
-      </c>
-      <c r="D62" t="s">
-        <v>14</v>
-      </c>
-      <c r="E62" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>131</v>
-      </c>
-      <c r="B63" t="s">
-        <v>12</v>
-      </c>
-      <c r="C63" t="s">
-        <v>134</v>
-      </c>
-      <c r="D63" t="s">
-        <v>14</v>
-      </c>
-      <c r="E63" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>131</v>
-      </c>
-      <c r="B64" t="s">
-        <v>12</v>
-      </c>
-      <c r="C64" t="s">
-        <v>135</v>
-      </c>
-      <c r="D64" t="s">
-        <v>14</v>
-      </c>
-      <c r="E64" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
dashboard: an event limit that binds on the ordinary case is set wrong
EVENT_CAP was 500 per chunk. With the chunk-loop fix in place, the default
whole-register document read 500 of the 1,054 events its projects hold,
so the coverage note printed "What moved is not a complete list" on every
document generated. The note was true, which is worse than if it had been
wrong: a limit that binds on the ordinary case is not a runaway guard, it
is a silent ceiling that had just learned to speak.

2,000. Above everything this corpus holds, still bounded, and stated in
the coverage note if it ever binds.

The event-read audit now reports COMPLETE: all 1,054 events the database
holds for a 265-project document reach it, including 369 from the 115
projects past the chunk boundary that the single-chunk read returned zero
of by construction.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/e2e/shots/documents/full-report.xlsx
+++ b/dashboard/e2e/shots/documents/full-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="720" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="249">
   <si>
     <t>Market intelligence report</t>
   </si>
@@ -737,6 +737,9 @@
   </si>
   <si>
     <t>This document describes the 15 most significant projects in scope. Every project in scope is described.</t>
+  </si>
+  <si>
+    <t>3 projects described above have a one-line description on our register that is not printed here. Those lines were written by a model reading the filings rather than quoted from one, so there is no document to cite for them and they are not offered as Philip's assessment either. The filings under each entry are unaffected.</t>
   </si>
   <si>
     <t>2 projects in scope are not named in this document because our capture holds no published name for them - only the agenda line the matter was filed under, which is the instrument rather than the project. They are on the register and can be named by hand. By market: Phoenix (2).</t>
@@ -1135,7 +1138,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F126"/>
+  <dimension ref="A1:F127"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -3555,6 +3558,26 @@
         <v>13</v>
       </c>
     </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>237</v>
+      </c>
+      <c r="B127" t="s">
+        <v>13</v>
+      </c>
+      <c r="C127" t="s">
+        <v>14</v>
+      </c>
+      <c r="D127" t="s">
+        <v>248</v>
+      </c>
+      <c r="E127" t="s">
+        <v>13</v>
+      </c>
+      <c r="F127" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
harness: the shot documents carry the scale block
Regenerated by the suite against the new build, so the read-back
artifacts in e2e/shots/documents are the documents this code produces
rather than the ones the previous build did.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/e2e/shots/documents/full-report.xlsx
+++ b/dashboard/e2e/shots/documents/full-report.xlsx
@@ -19,13 +19,13 @@
     <t>Prepared for Simtec Attractions by Philip Kwong</t>
   </si>
   <si>
-    <t>Geography: Altamonte Springs, Anaheim, Atlanta, Bonita Springs, Central Florida Tourism Oversight District, Clark County, Kissimmee, Lake Buena Vista, Las Vegas, Miami-Dade County, Nashville, Oakland, Phoenix, San Antonio, South Florida, Walt Disney World</t>
+    <t>Geography: United States &gt; Altamonte Springs, Anaheim, Bonita Springs, Central Florida Tourism Oversight District, Clark County, Kissimmee, Lake Buena Vista, Las Vegas, Miami-Dade County, Nashville, Oakland, Phoenix, San Antonio, South Florida, Walt Disney World</t>
   </si>
   <si>
     <t>Period: July 2026</t>
   </si>
   <si>
-    <t>Filters: dormant excluded | context records included | stage: hearing scheduled | stage: approved | stage: permitted | stage: under construction | venue: Theme Park | venue: Amusement Park | venue: Waterpark | venue: Family Entertainment Center | venue: Museum | venue: Aquarium | venue: Science Center | venue: Heritage/Cultural Site | venue: Arena/Stadium | venue: Integrated Resort | venue: Casino/Gaming | venue: Entertainment District | venue: Entertainment Destination | venue: Mixed-Use Development</t>
+    <t>Filters: dormant excluded | context records included | stage: hearing scheduled | stage: approved | stage: permitted | stage: under construction | venue: Theme Park | venue: Amusement Park | venue: Family Entertainment Center | venue: Museum | venue: Aquarium | venue: Science Center | venue: Heritage/Cultural Site | venue: Integrated Resort | venue: Casino/Gaming | venue: Entertainment District | venue: Entertainment Destination | venue: Mixed-Use Development</t>
   </si>
   <si>
     <t>Basis: 0 projects, 0 records</t>
@@ -58,13 +58,13 @@
     <t>ASSESSMENT</t>
   </si>
   <si>
-    <t>This report covers Altamonte Springs, Anaheim, Atlanta, Bonita Springs, Central Florida Tourism Oversight District, Clark County, Kissimmee, Lake Buena Vista, Las Vegas, Miami-Dade County, Nashville, Oakland, Phoenix, San Antonio, South Florida, Walt Disney World for July 2026. It is drawn from 0 projects and 0 captured records. Of those projects, 0 are described in full, selected by significance. 1 project whose every record has been dismissed is excluded entirely, because it has no filing to cite. Anything outside that geography or period is not covered here.</t>
+    <t>This report covers United States &gt; Altamonte Springs, Anaheim, Bonita Springs, Central Florida Tourism Oversight District, Clark County, Kissimmee, Lake Buena Vista, Las Vegas, Miami-Dade County, Nashville, Oakland, Phoenix, San Antonio, South Florida, Walt Disney World for July 2026. It is drawn from 0 projects and 0 captured records. Of those projects, 0 are described in full, selected by significance. 1 project whose every record has been dismissed is excluded entirely, because it has no filing to cite. Anything outside that geography or period is not covered here.</t>
   </si>
   <si>
     <t>Coverage note</t>
   </si>
   <si>
-    <t>Coverage is limited to Altamonte Springs, Anaheim, Atlanta, Bonita Springs, Central Florida Tourism Oversight District, Clark County, Kissimmee, Lake Buena Vista, Las Vegas, Miami-Dade County, Nashville, Oakland, Phoenix, San Antonio, South Florida, Walt Disney World. Projects outside it exist in our register and are not reported here.</t>
+    <t>Coverage is limited to United States &gt; Altamonte Springs, Anaheim, Bonita Springs, Central Florida Tourism Oversight District, Clark County, Kissimmee, Lake Buena Vista, Las Vegas, Miami-Dade County, Nashville, Oakland, Phoenix, San Antonio, South Florida, Walt Disney World. Projects outside it exist in our register and are not reported here.</t>
   </si>
   <si>
     <t>The period is July 2026. Activity outside it is not included even where it concerns the same project.</t>

</xml_diff>

<commit_message>
shots: regenerate the artefacts from the green run
71 passed. referral-brief.pdf now carries the coverage note section, which is
the artefact evidence for the referral change rather than a claim about it.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/e2e/shots/documents/full-report.xlsx
+++ b/dashboard/e2e/shots/documents/full-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="176">
   <si>
     <t>Market intelligence report</t>
   </si>
@@ -100,162 +100,162 @@
     <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3618#item-h84e398be28a0</t>
   </si>
   <si>
-    <t>Disneyland Resort: Determination that the property owner has complied in good faith with the terms and conditions of the First Amended and Restated Development Agreement No. 96-01 for the 2025-2026 review period for the Disneyland Resort Project</t>
+    <t>Disneyland Resort: Determine compliance in good faith with the terms and conditions of First Amended and Restated Development Agreement No. 96-01 for the 2025-2026 review period</t>
   </si>
   <si>
     <t>2026-06-22 | Anaheim</t>
   </si>
   <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3636#item-h5cf18daa4ec3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Approve the Cooperative Agreement with Walt Disney Parks and Resorts U.S., INC., in the amount estimated at $10,030,000, for funding, design...</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3511#item-h2d4a3a6c3f2a</t>
+  </si>
+  <si>
+    <t>CFTOD / Walt Disney World: Approve the First Amendment to Roadway Expansion Land Dedication and Reimbursement Agreement and authorize the District Administrator or her designee to execute same</t>
+  </si>
+  <si>
+    <t>2026-01-23 | Central Florida Tourism Oversight District</t>
+  </si>
+  <si>
+    <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/1-23-2026-BOS-Agenda-Packet-FINALcs.pdf#item-6.2-p12</t>
+  </si>
+  <si>
+    <t>Platinum Triangle / PT Metro: Establish new development timeframes and performance time schedule for Development Agreement No. 2005-00008</t>
+  </si>
+  <si>
+    <t>2026-01-26 | Anaheim</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3560#item-h9f77764dd1e5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Development agreement no. 2005-00008 Addendum no. 4 To platinum triangle expansion project mitigation monitoring plan no. 321 Applicant : PT Metro, LLC and Joey Caucas; 20 Enterprise, Suite #125...</t>
+  </si>
+  <si>
+    <t>Entertainment/Attractions</t>
+  </si>
+  <si>
+    <t>OCVibe</t>
+  </si>
+  <si>
+    <t>Approve Cooperative Agreement No. 12-0876, in substantial form, with Caltrans for design (plans, specifications, and estimates) services for the Northbound SR-57 Off-Ramp to Katella Avenue...</t>
+  </si>
+  <si>
+    <t>Anaheim | approved</t>
+  </si>
+  <si>
+    <t>Records show 4 filings and 4 press reports between 2026-02-06 and 2026-07-13.</t>
+  </si>
+  <si>
+    <t>Party: Anaheim Real Estate Partners, LLC</t>
+  </si>
+  <si>
+    <t>applicant | No phone or email in the record.</t>
+  </si>
+  <si>
+    <t>Party: Anaheim Real Estate Partners, LLC, TS Anaheim, LLC and FCD, LLC (OCVIBE)</t>
+  </si>
+  <si>
+    <t>Party: Lisandro Orozco</t>
+  </si>
+  <si>
+    <t>presented by; contact named in the record | lorozco@anaheim.net</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_45b322ae69423ed7f4d96ffe8e8de725.pdf&amp;view=1#item-h9fe8d90cfc0b</t>
+  </si>
+  <si>
+    <t>Party: City of Anaheim</t>
+  </si>
+  <si>
+    <t>presented by | No phone or email in the record.</t>
+  </si>
+  <si>
+    <t>https://ceqanet.lci.ca.gov/Project/2004121045</t>
+  </si>
+  <si>
+    <t>Party: Stacy Tran</t>
+  </si>
+  <si>
+    <t>presented by; contact named in the record | STran@anaheim.net</t>
+  </si>
+  <si>
+    <t>https://www.anaheim.net/DocumentCenter/View/66931/Planning-Commission-Action-Agenda---10202025#item-h6dc7e70418cc</t>
+  </si>
+  <si>
+    <t>2026-02-06. OCVibe Residential Phase I</t>
+  </si>
+  <si>
+    <t>Players: City of Anaheim (presented by)</t>
+  </si>
+  <si>
+    <t>2026-04-20. Approve Amendment No. 2 to Bond Purchase Agreement between the City of Anaheim, the Public Financing Authority, and JP Morgan amending the scheduled completion date to no later than June 25, 2027 for the parking decks associated with the OCVibe Project; and authorize the Finance Director to execute the amendment</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3606#item-h11f1fc13fc80</t>
+  </si>
+  <si>
+    <t>2026-05-05. OCVibe | The new heart of Orange County</t>
+  </si>
+  <si>
+    <t>https://www.ocvibe.com/news/ocvibe-and-award-winning-art-and-design-studio-futureforms-unveil-plans-for-historic-arts-program-in-southern-california</t>
+  </si>
+  <si>
+    <t>2026-05-11. Approve Cooperative Agreement No. 12-0876 with Caltrans for design services and Cooperative Agreement No. 12-0877 with Caltrans for right-of-way services for SR-57 off-ramps</t>
+  </si>
+  <si>
+    <t>2026-05-17. Southern California gets $4B mega music venue in giant ...</t>
+  </si>
+  <si>
+    <t>https://nypost.com/2026/05/18/lifestyle/southern-california-lands-mega-venue-in-new-entertainment-district/</t>
+  </si>
+  <si>
+    <t>2026-05-31. First Phase of $4B OCVibe Takes Shape</t>
+  </si>
+  <si>
+    <t>https://www.ocbj.com/oc-homepage/first-phase-of-4b-ocvibe-takes-shape/</t>
+  </si>
+  <si>
+    <t>2026-06-22. 2525 E Katella Ave, Anaheim, CA 92806 - The Weave ...</t>
+  </si>
+  <si>
+    <t>https://www.loopnet.com/Listing/2525-E-Katella-Ave-Anaheim-CA/29241061/</t>
+  </si>
+  <si>
+    <t>2026-07-13. Determine on the basis of the evidence submitted by Anaheim Real Estate Partners, LLC, TS Anaheim, LLC, and FCD, LLC (OCVibe), that the property owner has complied in good faith with the terms and conditions of Amended and Restated Development Agreement No...</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3646#item-heb30443bfb8b</t>
+  </si>
+  <si>
+    <t>Disneyland Resort</t>
+  </si>
+  <si>
+    <t>Approve the Cooperative Agreement with Walt Disney Parks and Resorts U.S., INC., in the amount estimated at $10,030,000, for funding, design...</t>
+  </si>
+  <si>
+    <t>Records show 4 filings on the first amended and restated development agreement between 2024-05-08 and 2026-06-22.</t>
+  </si>
+  <si>
+    <t>Party: Walt Disney Parks and Resorts U.S., Inc.</t>
+  </si>
+  <si>
+    <t>Party: Disneyland</t>
+  </si>
+  <si>
+    <t>https://ceqanet.lci.ca.gov/Project/2021100402</t>
+  </si>
+  <si>
+    <t>Party: Walt Disney Parks and Resorts US, Inc.</t>
+  </si>
+  <si>
     <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_5713ee926e19136cdccede9cc8a3ce47.pdf&amp;view=1#item-h72954c9ae56e</t>
   </si>
   <si>
-    <t xml:space="preserve">   Approve the Cooperative Agreement with Walt Disney Parks and Resorts U.S., INC., in the amount estimated at $10,030,000, for funding, design...</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3511#item-h2d4a3a6c3f2a</t>
-  </si>
-  <si>
-    <t>CFTOD / Walt Disney World: Approve the First Amendment to Roadway Expansion Land Dedication and Reimbursement Agreement and authorize the District Administrator or her designee to execute same</t>
-  </si>
-  <si>
-    <t>2026-01-23 | Central Florida Tourism Oversight District</t>
-  </si>
-  <si>
-    <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/1-23-2026-BOS-Agenda-Packet-FINALcs.pdf#item-6.2-p12</t>
-  </si>
-  <si>
-    <t>Platinum Triangle / PT Metro: Establish new development timeframes and performance time schedule for Development Agreement No. 2005-00008</t>
-  </si>
-  <si>
-    <t>2026-01-26 | Anaheim</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3560#item-h9f77764dd1e5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Development agreement no. 2005-00008 Addendum no. 4 To platinum triangle expansion project mitigation monitoring plan no. 321 Applicant : PT Metro, LLC and Joey Caucas; 20 Enterprise, Suite #125...</t>
-  </si>
-  <si>
-    <t>Entertainment/Attractions</t>
-  </si>
-  <si>
-    <t>OCVibe</t>
-  </si>
-  <si>
-    <t>Approve Cooperative Agreement No. 12-0876, in substantial form, with Caltrans for design (plans, specifications, and estimates) services for the Northbound SR-57 Off-Ramp to Katella Avenue...</t>
-  </si>
-  <si>
-    <t>Anaheim | approved</t>
-  </si>
-  <si>
-    <t>Records show 4 filings and 4 press reports between 2026-02-06 and 2026-07-13.</t>
-  </si>
-  <si>
-    <t>Party: Anaheim Real Estate Partners, LLC</t>
-  </si>
-  <si>
-    <t>applicant | No phone or email in the record.</t>
-  </si>
-  <si>
-    <t>Party: Anaheim Real Estate Partners, LLC, TS Anaheim, LLC and FCD, LLC (OCVIBE)</t>
-  </si>
-  <si>
-    <t>Party: Lisandro Orozco</t>
-  </si>
-  <si>
-    <t>presented by; contact named in the record | lorozco@anaheim.net</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_45b322ae69423ed7f4d96ffe8e8de725.pdf&amp;view=1#item-h9fe8d90cfc0b</t>
-  </si>
-  <si>
-    <t>Party: City of Anaheim</t>
-  </si>
-  <si>
-    <t>presented by | No phone or email in the record.</t>
-  </si>
-  <si>
-    <t>https://ceqanet.lci.ca.gov/Project/2004121045</t>
-  </si>
-  <si>
-    <t>Party: Stacy Tran</t>
-  </si>
-  <si>
-    <t>presented by; contact named in the record | STran@anaheim.net</t>
-  </si>
-  <si>
-    <t>https://www.anaheim.net/DocumentCenter/View/66931/Planning-Commission-Action-Agenda---10202025#item-h6dc7e70418cc</t>
-  </si>
-  <si>
-    <t>2026-02-06. OCVibe Residential Phase I</t>
-  </si>
-  <si>
-    <t>Players: City of Anaheim (presented by)</t>
-  </si>
-  <si>
-    <t>2026-04-20. Approve Amendment No. 2 to Bond Purchase Agreement between the City of Anaheim, the Public Financing Authority, and JP Morgan amending the scheduled completion date to no later than June 25, 2027 for the parking decks associated with the OCVibe Project; and authorize the Finance Director to execute the amendment</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3606#item-h11f1fc13fc80</t>
-  </si>
-  <si>
-    <t>2026-05-05. OCVibe | The new heart of Orange County</t>
-  </si>
-  <si>
-    <t>https://www.ocvibe.com/news/ocvibe-and-award-winning-art-and-design-studio-futureforms-unveil-plans-for-historic-arts-program-in-southern-california</t>
-  </si>
-  <si>
-    <t>2026-05-11. Approve Cooperative Agreement No. 12-0876 with Caltrans for design services and Cooperative Agreement No. 12-0877 with Caltrans for right-of-way services for SR-57 off-ramps</t>
-  </si>
-  <si>
-    <t>2026-05-17. Southern California gets $4B mega music venue in giant ...</t>
-  </si>
-  <si>
-    <t>https://nypost.com/2026/05/18/lifestyle/southern-california-lands-mega-venue-in-new-entertainment-district/</t>
-  </si>
-  <si>
-    <t>2026-05-31. First Phase of $4B OCVibe Takes Shape</t>
-  </si>
-  <si>
-    <t>https://www.ocbj.com/oc-homepage/first-phase-of-4b-ocvibe-takes-shape/</t>
-  </si>
-  <si>
-    <t>2026-06-22. 2525 E Katella Ave, Anaheim, CA 92806 - The Weave ...</t>
-  </si>
-  <si>
-    <t>https://www.loopnet.com/Listing/2525-E-Katella-Ave-Anaheim-CA/29241061/</t>
-  </si>
-  <si>
-    <t>2026-07-13. Determine on the basis of the evidence submitted by Anaheim Real Estate Partners, LLC, TS Anaheim, LLC, and FCD, LLC (OCVibe), that the property owner has complied in good faith with the terms and conditions of Amended and Restated Development Agreement No...</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3646#item-heb30443bfb8b</t>
-  </si>
-  <si>
-    <t>Disneyland Resort</t>
-  </si>
-  <si>
-    <t>Approve the Cooperative Agreement with Walt Disney Parks and Resorts U.S., INC., in the amount estimated at $10,030,000, for funding, design...</t>
-  </si>
-  <si>
-    <t>Records show 4 filings on the first amended and restated development agreement between 2024-05-08 and 2026-06-22.</t>
-  </si>
-  <si>
-    <t>Party: Walt Disney Parks and Resorts U.S., Inc.</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3636#item-h5cf18daa4ec3</t>
-  </si>
-  <si>
-    <t>Party: Disneyland</t>
-  </si>
-  <si>
-    <t>https://ceqanet.lci.ca.gov/Project/2021100402</t>
-  </si>
-  <si>
-    <t>Party: Walt Disney Parks and Resorts US, Inc.</t>
-  </si>
-  <si>
     <t>2024-05-08. DisneylandForward Project</t>
   </si>
   <si>
@@ -436,37 +436,58 @@
     <t>Party: Kulik River Capital, LLC</t>
   </si>
   <si>
+    <t>https://clark.legistar.com/Legislation.aspx#matter-110427</t>
+  </si>
+  <si>
+    <t>Party: Nancy Amundsen</t>
+  </si>
+  <si>
+    <t>representative; contact named in the record | Brown, Brown, &amp; Premsrirut | 520 S. 4th Street, Las Vegas, NV 89101 | No phone or email in the record.</t>
+  </si>
+  <si>
+    <t>Party: Eli Applebaum</t>
+  </si>
+  <si>
+    <t>https://www.mundovideo.com.co/en/america/ballys-chicago-and-skyvue-casino-plans-to-advance-in-illinois-and-nevada/</t>
+  </si>
+  <si>
+    <t>2026-05-26. Vacate and abandon easements of interest to Clark County located between Mandalay Bay Road and Four Seasons Drive, and Las Vegas Boulevard South and Haven Street; and a portion of a right-of-way being Mandalay Bay Road located between Las Vegas Boulevard South and Haven Street</t>
+  </si>
+  <si>
+    <t>VS-26-0218</t>
+  </si>
+  <si>
+    <t>https://www.clarkcountynv.gov/adobe/assets/urn:aaid:aem:bcdf1925-6c37-4308-b6f6-c718c78c9183/original/as/Paradise-Minutes-052626.pdf#item-vs-26-0218</t>
+  </si>
+  <si>
+    <t>2026-05-26. Tentative map approval for 1 commercial lot on 11.95 acres in a CR (Commercial Resort) Zone within the Airport Environs (AE-60) Overlay</t>
+  </si>
+  <si>
+    <t>TM-26-500056</t>
+  </si>
+  <si>
+    <t>2026-07-21. Holdover tentative map</t>
+  </si>
+  <si>
+    <t>TM-26-500056 | 11.95 acres | Contact: Nancy Amundsen, Brown, Brown, &amp; Premsrirut. No phone or email in the record.</t>
+  </si>
+  <si>
     <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110427</t>
   </si>
   <si>
-    <t>Party: Nancy Amundsen</t>
-  </si>
-  <si>
-    <t>representative; contact named in the record | Brown, Brown, &amp; Premsrirut | 520 S. 4th Street, Las Vegas, NV 89101 | No phone or email in the record.</t>
-  </si>
-  <si>
-    <t>Party: Eli Applebaum</t>
-  </si>
-  <si>
-    <t>https://www.mundovideo.com.co/en/america/ballys-chicago-and-skyvue-casino-plans-to-advance-in-illinois-and-nevada/</t>
-  </si>
-  <si>
-    <t>2026-05-26. Vacate and abandon easements of interest to Clark County located between Mandalay Bay Road and Four Seasons Drive, and Las Vegas Boulevard South and Haven Street; and a portion of a right-of-way being Mandalay Bay Road located between Las Vegas Boulevard South and Haven Street</t>
-  </si>
-  <si>
-    <t>VS-26-0218</t>
-  </si>
-  <si>
-    <t>https://www.clarkcountynv.gov/adobe/assets/urn:aaid:aem:bcdf1925-6c37-4308-b6f6-c718c78c9183/original/as/Paradise-Minutes-052626.pdf#item-vs-26-0218</t>
-  </si>
-  <si>
-    <t>2026-05-26. Use permits to expand gaming enterprise district, construct resort hotel, and construct recreational facility; waiver of development standards; design review</t>
-  </si>
-  <si>
-    <t>UC-26-0219</t>
-  </si>
-  <si>
-    <t>https://www.clarkcountynv.gov/adobe/assets/urn:aaid:aem:bcdf1925-6c37-4308-b6f6-c718c78c9183/original/as/Paradise-Minutes-052626.pdf#item-uc-26-0219</t>
+    <t>2026-07-21. Vacate and abandon easements of interest to Clark County located between Mandalay Bay Road and Four Seasons Drive, and Las Vegas Boulevard South and Haven Street; and a portion of a right-of-way being Mandalay Bay Road located between Las Vegas Boulevard South and Haven Street within Paradise</t>
+  </si>
+  <si>
+    <t>VS-26-0218 | Contact: Nancy Amundsen, Brown, Brown, &amp; Premsrirut. No phone or email in the record.</t>
+  </si>
+  <si>
+    <t>https://clark.legistar.com/Legislation.aspx#matter-110425</t>
+  </si>
+  <si>
+    <t>2026-07-21. Resort project replacing failed Las Vegas Strip observation ...</t>
+  </si>
+  <si>
+    <t>https://news3lv.com/news/local/resort-project-skyvue-failed-las-vegas-strip-observation-wheel-clark-county-commission-zoning-approval</t>
   </si>
   <si>
     <t>2026-07-21. Holdover use permits to expand the gaming enterprise district, resort hotel, and recreational facility; Waiver of development standards to allow non-standard improvements in the right-of-way; Design review for a proposed resort hotel and recreational facility</t>
@@ -478,27 +499,6 @@
     <t>https://clark.legistar.com/Legislation.aspx#matter-110426</t>
   </si>
   <si>
-    <t>2026-07-21. Vacate and abandon easements of interest to Clark County located between Mandalay Bay Road and Four Seasons Drive, and Las Vegas Boulevard South and Haven Street; and a portion of a right-of-way being Mandalay Bay Road located between Las Vegas Boulevard South and Haven Street within Paradise</t>
-  </si>
-  <si>
-    <t>VS-26-0218 | Contact: Nancy Amundsen, Brown, Brown, &amp; Premsrirut. No phone or email in the record.</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/Legislation.aspx#matter-110425</t>
-  </si>
-  <si>
-    <t>2026-07-21. Resort project replacing failed Las Vegas Strip observation ...</t>
-  </si>
-  <si>
-    <t>https://news3lv.com/news/local/resort-project-skyvue-failed-las-vegas-strip-observation-wheel-clark-county-commission-zoning-approval</t>
-  </si>
-  <si>
-    <t>2026-07-21. Holdover tentative map</t>
-  </si>
-  <si>
-    <t>TM-26-500056 | 11.95 acres | Contact: Nancy Amundsen, Brown, Brown, &amp; Premsrirut. No phone or email in the record.</t>
-  </si>
-  <si>
     <t>2026-07-23. Las Vegas Approves Heart-Shaped Casino on SkyVue Site</t>
   </si>
   <si>
@@ -506,6 +506,9 @@
   </si>
   <si>
     <t>2026-07-24. Las Vegas Topic Kulik River Capital</t>
+  </si>
+  <si>
+    <t>Watch list</t>
   </si>
   <si>
     <t>Coverage note</t>
@@ -916,7 +919,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1533,7 +1536,7 @@
         <v>47</v>
       </c>
       <c r="F36" t="s">
-        <v>77</v>
+        <v>31</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -1547,13 +1550,13 @@
         <v>21</v>
       </c>
       <c r="D37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E37" t="s">
         <v>47</v>
       </c>
       <c r="F37" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -1567,13 +1570,13 @@
         <v>21</v>
       </c>
       <c r="D38" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E38" t="s">
         <v>47</v>
       </c>
       <c r="F38" t="s">
-        <v>31</v>
+        <v>80</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -1593,7 +1596,7 @@
         <v>53</v>
       </c>
       <c r="F39" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -1613,7 +1616,7 @@
         <v>82</v>
       </c>
       <c r="F40" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -1673,7 +1676,7 @@
         <v>13</v>
       </c>
       <c r="F43" t="s">
-        <v>77</v>
+        <v>31</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -2213,7 +2216,7 @@
         <v>150</v>
       </c>
       <c r="F70" t="s">
-        <v>151</v>
+        <v>23</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
@@ -2227,13 +2230,13 @@
         <v>21</v>
       </c>
       <c r="D71" t="s">
+        <v>151</v>
+      </c>
+      <c r="E71" t="s">
         <v>152</v>
       </c>
-      <c r="E71" t="s">
+      <c r="F71" t="s">
         <v>153</v>
-      </c>
-      <c r="F71" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -2247,13 +2250,13 @@
         <v>21</v>
       </c>
       <c r="D72" t="s">
+        <v>154</v>
+      </c>
+      <c r="E72" t="s">
         <v>155</v>
       </c>
-      <c r="E72" t="s">
+      <c r="F72" t="s">
         <v>156</v>
-      </c>
-      <c r="F72" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
@@ -2267,13 +2270,13 @@
         <v>17</v>
       </c>
       <c r="D73" t="s">
+        <v>157</v>
+      </c>
+      <c r="E73" t="s">
+        <v>13</v>
+      </c>
+      <c r="F73" t="s">
         <v>158</v>
-      </c>
-      <c r="E73" t="s">
-        <v>13</v>
-      </c>
-      <c r="F73" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -2287,13 +2290,13 @@
         <v>21</v>
       </c>
       <c r="D74" t="s">
+        <v>159</v>
+      </c>
+      <c r="E74" t="s">
         <v>160</v>
       </c>
-      <c r="E74" t="s">
+      <c r="F74" t="s">
         <v>161</v>
-      </c>
-      <c r="F74" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
@@ -2344,21 +2347,21 @@
         <v>13</v>
       </c>
       <c r="C77" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D77" t="s">
-        <v>166</v>
+        <v>18</v>
       </c>
       <c r="E77" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F77" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B78" t="s">
         <v>13</v>
@@ -2378,7 +2381,7 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B79" t="s">
         <v>13</v>
@@ -2398,7 +2401,7 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B80" t="s">
         <v>13</v>
@@ -2418,7 +2421,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B81" t="s">
         <v>13</v>
@@ -2438,7 +2441,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B82" t="s">
         <v>13</v>
@@ -2458,7 +2461,7 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B83" t="s">
         <v>13</v>
@@ -2478,7 +2481,7 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B84" t="s">
         <v>13</v>
@@ -2498,7 +2501,7 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B85" t="s">
         <v>13</v>
@@ -2513,6 +2516,26 @@
         <v>13</v>
       </c>
       <c r="F85" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>166</v>
+      </c>
+      <c r="B86" t="s">
+        <v>13</v>
+      </c>
+      <c r="C86" t="s">
+        <v>14</v>
+      </c>
+      <c r="D86" t="s">
+        <v>175</v>
+      </c>
+      <c r="E86" t="s">
+        <v>13</v>
+      </c>
+      <c r="F86" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
shots: regenerate the artefacts from the 71 of 71 run
Every document and screenshot rebuilt by the run that took the suite from 70 of
71 to 71 of 71. The referral brief is the one worth reading: it now carries the
press-named role rather than "contact named in the record", and it is the artefact
the six blemishes were read out of.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/e2e/shots/documents/full-report.xlsx
+++ b/dashboard/e2e/shots/documents/full-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="178">
   <si>
     <t>Market intelligence report</t>
   </si>
@@ -25,7 +25,7 @@
     <t>Period: July 2026</t>
   </si>
   <si>
-    <t>Filters: dormant excluded | context records included | stage: hearing scheduled | stage: approved | stage: permitted | stage: under construction | venue: Theme Park | venue: Amusement Park | venue: Family Entertainment Center | venue: Museum | venue: Aquarium | venue: Science Center | venue: Heritage/Cultural Site | venue: Integrated Resort | venue: Casino/Gaming | venue: Entertainment District | venue: Entertainment Destination | venue: Mixed-Use Development</t>
+    <t>Filters: dormant excluded | context records included | stage: filed | stage: hearing scheduled | stage: approved | stage: permitted | stage: under construction | venue: Theme Park | venue: Amusement Park | venue: Family Entertainment Center | venue: Museum | venue: Aquarium | venue: Science Center | venue: Heritage/Cultural Site | venue: Integrated Resort | venue: Casino/Gaming | venue: Entertainment District | venue: Entertainment Destination | venue: Mixed-Use Development</t>
   </si>
   <si>
     <t>Basis: 5 projects, 53 records</t>
@@ -58,12 +58,30 @@
     <t>ASSESSMENT</t>
   </si>
   <si>
-    <t>This report covers United States &gt; Altamonte Springs, Anaheim, Bonita Springs, Central Florida Tourism Oversight District, Clark County, Kissimmee, Lake Buena Vista, Las Vegas, Miami-Dade County, Nashville, Oakland, Phoenix, San Antonio, South Florida, Walt Disney World for July 2026. It is drawn from 5 projects and 53 captured records. Of those projects, 5 are described in full, selected by significance. 9 projects this scope proposes are held out of this document because they have not been confirmed as part of Simtec Attractions' coverage. A scope is a proposal: it finds projects that look like a match, and each one is confirmed by hand on the register before it may be printed. Those projects are on the register, unconfirmed, and are not a statement that they do not belong here. Anything outside that geography or period is not covered here.</t>
+    <t>This report covers United States &gt; Altamonte Springs, Anaheim, Bonita Springs, Central Florida Tourism Oversight District, Clark County, Kissimmee, Lake Buena Vista, Las Vegas, Miami-Dade County, Nashville, Oakland, Phoenix, San Antonio, South Florida, Walt Disney World for July 2026. It is drawn from 5 projects and 53 captured records. Of those projects, 5 are described in full, selected by significance. 40 projects this scope proposes are held out of this document because they have not been confirmed as part of Simtec Attractions' coverage. A scope is a proposal: it finds projects that look like a match, and each one is confirmed by hand on the register before it may be printed. Those projects are on the register, unconfirmed, and are not a statement that they do not belong here. Anything outside that geography or period is not covered here.</t>
   </si>
   <si>
     <t>Headline finds</t>
   </si>
   <si>
+    <t>RECORD</t>
+  </si>
+  <si>
+    <t>OCVibe: Determine on the basis of the evidence submitted by Anaheim Real Estate Partners, LLC, TS Anaheim, LLC, and FCD, LLC (OCVibe), that the property owner has complied in good faith with the terms and conditions of Amended and Restated Development Agreement No...</t>
+  </si>
+  <si>
+    <t>2026-07-13 | Anaheim</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3646#item-heb30443bfb8b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Approve Cooperative Agreement No. 12-0876, in substantial form, with Caltrans for design (plans, specifications, and estimates) services for the Northbound SR-57 Off-Ramp to Katella Avenue...</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3618#item-h84e398be28a0</t>
+  </si>
+  <si>
     <t>PRESS</t>
   </si>
   <si>
@@ -76,94 +94,79 @@
     <t>https://news3lv.com/topic/Kulik%20River%20Capital</t>
   </si>
   <si>
-    <t>RECORD</t>
-  </si>
-  <si>
     <t xml:space="preserve">   Kulik river capital, LLC: Tentative map consisting of 1 commercial lot on 11.95 acres in a CR (Commercial Resort) Zone within the Airport Environs (AE-60) Overlay.</t>
   </si>
   <si>
     <t>https://www.clarkcountynv.gov/adobe/assets/urn:aaid:aem:bcdf1925-6c37-4308-b6f6-c718c78c9183/original/as/Paradise-Minutes-052626.pdf#item-tm-26-500056</t>
   </si>
   <si>
-    <t>OCVibe: Determination that property owner has complied in good faith with the terms and conditions of Amended and Restated Development Agreement No. 2020-00004 for the 2025-2026 review period for the OCVibe Site Master Plan project</t>
-  </si>
-  <si>
-    <t>2026-07-13 | Anaheim</t>
+    <t>Disneyland Resort: Determine compliance in good faith with the terms and conditions of First Amended and Restated Development Agreement No. 96-01 for the 2025-2026 review period</t>
+  </si>
+  <si>
+    <t>2026-06-22 | Anaheim</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3636#item-h5cf18daa4ec3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Approve the Cooperative Agreement with Walt Disney Parks and Resorts U.S., INC., in the amount estimated at $10,030,000, for funding, design...</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3511#item-h2d4a3a6c3f2a</t>
+  </si>
+  <si>
+    <t>CFTOD / Walt Disney World: Approve the First Amendment to Roadway Expansion Land Dedication and Reimbursement Agreement and authorize the District Administrator or her designee to execute same</t>
+  </si>
+  <si>
+    <t>2026-01-23 | Central Florida Tourism Oversight District</t>
+  </si>
+  <si>
+    <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/1-23-2026-BOS-Agenda-Packet-FINALcs.pdf#item-6.2-p12</t>
+  </si>
+  <si>
+    <t>Platinum Triangle / PT Metro: Establish new development timeframes and performance time schedule for Development Agreement No. 2005-00008</t>
+  </si>
+  <si>
+    <t>2026-01-26 | Anaheim</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3560#item-h9f77764dd1e5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Development agreement no. 2005-00008 Addendum no. 4 To platinum triangle expansion project mitigation monitoring plan no. 321 Applicant : PT Metro, LLC and Joey Caucas; 20 Enterprise, Suite #125...</t>
+  </si>
+  <si>
+    <t>Entertainment/Attractions</t>
+  </si>
+  <si>
+    <t>OCVibe</t>
+  </si>
+  <si>
+    <t>Approve Cooperative Agreement No. 12-0876, in substantial form, with Caltrans for design (plans, specifications, and estimates) services for the Northbound SR-57 Off-Ramp to Katella Avenue...</t>
+  </si>
+  <si>
+    <t>Anaheim | approved</t>
+  </si>
+  <si>
+    <t>Records show 4 filings and 4 press reports between 2026-02-06 and 2026-07-13.</t>
+  </si>
+  <si>
+    <t>Party: Anaheim Real Estate Partners, LLC</t>
+  </si>
+  <si>
+    <t>applicant | No phone or email in the record.</t>
+  </si>
+  <si>
+    <t>Party: Anaheim Real Estate Partners, LLC, TS Anaheim, LLC and FCD, LLC (OCVIBE)</t>
   </si>
   <si>
     <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_7f2f654f7555addc70231de198fa22d9.pdf&amp;view=1#item-h9f002fc7dbca</t>
   </si>
   <si>
-    <t xml:space="preserve">   Approve Cooperative Agreement No. 12-0876, in substantial form, with Caltrans for design (plans, specifications, and estimates) services for the Northbound SR-57 Off-Ramp to Katella Avenue...</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3618#item-h84e398be28a0</t>
-  </si>
-  <si>
-    <t>Disneyland Resort: Determine compliance in good faith with the terms and conditions of First Amended and Restated Development Agreement No. 96-01 for the 2025-2026 review period</t>
-  </si>
-  <si>
-    <t>2026-06-22 | Anaheim</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3636#item-h5cf18daa4ec3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Approve the Cooperative Agreement with Walt Disney Parks and Resorts U.S., INC., in the amount estimated at $10,030,000, for funding, design...</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3511#item-h2d4a3a6c3f2a</t>
-  </si>
-  <si>
-    <t>CFTOD / Walt Disney World: Approve the First Amendment to Roadway Expansion Land Dedication and Reimbursement Agreement and authorize the District Administrator or her designee to execute same</t>
-  </si>
-  <si>
-    <t>2026-01-23 | Central Florida Tourism Oversight District</t>
-  </si>
-  <si>
-    <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/1-23-2026-BOS-Agenda-Packet-FINALcs.pdf#item-6.2-p12</t>
-  </si>
-  <si>
-    <t>Platinum Triangle / PT Metro: Establish new development timeframes and performance time schedule for Development Agreement No. 2005-00008</t>
-  </si>
-  <si>
-    <t>2026-01-26 | Anaheim</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3560#item-h9f77764dd1e5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Development agreement no. 2005-00008 Addendum no. 4 To platinum triangle expansion project mitigation monitoring plan no. 321 Applicant : PT Metro, LLC and Joey Caucas; 20 Enterprise, Suite #125...</t>
-  </si>
-  <si>
-    <t>Entertainment/Attractions</t>
-  </si>
-  <si>
-    <t>OCVibe</t>
-  </si>
-  <si>
-    <t>Approve Cooperative Agreement No. 12-0876, in substantial form, with Caltrans for design (plans, specifications, and estimates) services for the Northbound SR-57 Off-Ramp to Katella Avenue...</t>
-  </si>
-  <si>
-    <t>Anaheim | approved</t>
-  </si>
-  <si>
-    <t>Records show 4 filings and 4 press reports between 2026-02-06 and 2026-07-13.</t>
-  </si>
-  <si>
-    <t>Party: Anaheim Real Estate Partners, LLC</t>
-  </si>
-  <si>
-    <t>applicant | No phone or email in the record.</t>
-  </si>
-  <si>
-    <t>Party: Anaheim Real Estate Partners, LLC, TS Anaheim, LLC and FCD, LLC (OCVIBE)</t>
-  </si>
-  <si>
     <t>Party: Lisandro Orozco</t>
   </si>
   <si>
-    <t>presented by; contact named in the record | lorozco@anaheim.net</t>
+    <t>presented by; contact named in the filing | lorozco@anaheim.net</t>
   </si>
   <si>
     <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_45b322ae69423ed7f4d96ffe8e8de725.pdf&amp;view=1#item-h9fe8d90cfc0b</t>
@@ -181,7 +184,7 @@
     <t>Party: Stacy Tran</t>
   </si>
   <si>
-    <t>presented by; contact named in the record | STran@anaheim.net</t>
+    <t>presented by; contact named in the filing | STran@anaheim.net</t>
   </si>
   <si>
     <t>https://www.anaheim.net/DocumentCenter/View/66931/Planning-Commission-Action-Agenda---10202025#item-h6dc7e70418cc</t>
@@ -229,9 +232,6 @@
     <t>2026-07-13. Determine on the basis of the evidence submitted by Anaheim Real Estate Partners, LLC, TS Anaheim, LLC, and FCD, LLC (OCVibe), that the property owner has complied in good faith with the terms and conditions of Amended and Restated Development Agreement No...</t>
   </si>
   <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3646#item-heb30443bfb8b</t>
-  </si>
-  <si>
     <t>Disneyland Resort</t>
   </si>
   <si>
@@ -292,22 +292,22 @@
     <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/1-23-2026-BOS-Agenda-Packet-FINALcs.pdf#item-6.4-p146</t>
   </si>
   <si>
+    <t>Party: Katherine Luetzow</t>
+  </si>
+  <si>
+    <t>presented by | Director, Planning &amp; Engineering Department: Public Works | No phone or email in the record.</t>
+  </si>
+  <si>
     <t>Party: Craig Sandt</t>
   </si>
   <si>
     <t>presented by | Director of Construction Management | No phone or email in the record.</t>
   </si>
   <si>
-    <t>Party: Katherine Luetzow</t>
-  </si>
-  <si>
-    <t>presented by | Director, Planning &amp; Engineering Department, Public Works | No phone or email in the record.</t>
-  </si>
-  <si>
-    <t>2026-01-01. CFTOD 2045 Comprehensive Plan - theme park provisions (p.38)</t>
-  </si>
-  <si>
-    <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/2045-CFTOD-Comprehensive-Plan.pdf#plan-p38</t>
+    <t>2026-01-01. CFTOD 2045 Comprehensive Plan - recreation / tourist provisions (p.37)</t>
+  </si>
+  <si>
+    <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/2045-CFTOD-Comprehensive-Plan.pdf#plan-p37</t>
   </si>
   <si>
     <t>2026-01-23. Approve the First Amendment to Roadway Expansion Land Dedication and Reimbursement Agreement and authorize the District Administrator or her designee to execute same</t>
@@ -319,7 +319,7 @@
     <t>2026-01-23. Approve the District Administrator to execute a Non-exclusive temporary easement with permanent easement for underground communication lines</t>
   </si>
   <si>
-    <t>Players: Katherine Luetzow, Director, Planning &amp; Engineering Department, Public Works (presented by)</t>
+    <t>Players: Katherine Luetzow, Director, Planning &amp; Engineering Department: Public Works (presented by)</t>
   </si>
   <si>
     <t>Mixed-Use/Real Estate</t>
@@ -340,19 +340,22 @@
     <t>applicant | LLC and Joey Caucas | No phone or email in the record.</t>
   </si>
   <si>
+    <t>Party: City of Anaheim Planning Staff</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_2bfcbb0f5f83e7b944ef537de2b1fd4a.pdf&amp;view=1#item-ha13a91a5c59d</t>
+  </si>
+  <si>
     <t>Party: Christine Nguyen</t>
   </si>
   <si>
-    <t>presented by; contact named in the record | CNguyen2@anaheim.net | Also presenter on 2 other projects in our register: 2 in Anaheim.</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_2bfcbb0f5f83e7b944ef537de2b1fd4a.pdf&amp;view=1#item-ha13a91a5c59d</t>
+    <t>contact named in the filing | CNguyen2@anaheim.net | Also presenter on 2 other projects in our register: 2 in Anaheim.</t>
   </si>
   <si>
     <t>Party: Joey Caucas</t>
   </si>
   <si>
-    <t>contact named in the record | No phone or email in the record.</t>
+    <t>contact named in the filing | No phone or email in the record.</t>
   </si>
   <si>
     <t>2025-01-13. Adoption of Ordinance No. 6601 amending multiple chapters of Title 18 (Zoning) of the Anaheim Municipal Code and adjustments to multiple specific plans</t>
@@ -364,7 +367,7 @@
     <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3305#item-h9b4b4aa880b3</t>
   </si>
   <si>
-    <t>2025-03-23. City-initiated General Plan Amendments to update the General Plan Land Use and Circulation Elements, and adopt a new Environmental Justice Element; amendments to Title 18 (Zoning) of the Anaheim Municipal Code; Zoning Reclassification; amendments to the Platinum Triangle Master Land Use Plan...</t>
+    <t>2025-03-23. City-initiated General Plan Amendments to update the General Plan Land Use and Circulation Elements, adopt a new Environmental Justice Element, amend Title 18 (Zoning) of the Anaheim Municipal Code, reclassify zoning, and amend the Platinum Triangle Master Land Use Plan and specific plans...</t>
   </si>
   <si>
     <t>DEVELOPMENT APPLICATION No. 2021-00223</t>
@@ -391,10 +394,10 @@
     <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3398#item-h4c01cf1c0349</t>
   </si>
   <si>
-    <t>2025-08-10. General Plan Amendment to update the General Plan Land Use Element Table LU-2 (Residential Land Use Designations); amendments to Title 18 (Zoning) of the Anaheim Municipal Code modifying Chapters 18.06 (Multiple-Family Residential Zones), 18.12 (Mixed-Use Zone), and 18.52 (Housing Incentives)</t>
-  </si>
-  <si>
-    <t>DEVELOPMENT APPLICATION No. 2021-00223 | Players: Christine Nguyen (presented by) | Contact: Christine Nguyen. CNguyen2@anaheim.net.</t>
+    <t>2025-08-10. General Plan Amendment and Zoning Code amendments related to implementation of the Sixth Cycle Housing Element, including updates to General Plan Land Use Element Table LU-2 and amendments to Title 18 (Zoning) of the Anaheim Municipal Code</t>
+  </si>
+  <si>
+    <t>DEVELOPMENT APPLICATION No. 2021-00223 | Players: City of Anaheim Planning Staff (presented by) | Contact: Christine Nguyen. CNguyen2@anaheim.net.</t>
   </si>
   <si>
     <t>2025-08-11. Levying Special Taxes within City of Anaheim Community Facilities District No. 06-2 (Stadium Lofts) and Community Facilities District No. 08-1 (Platinum Triangle)</t>
@@ -427,7 +430,7 @@
     <t>Tentative map consisting of 1 commercial lot on 11.95 acres in a CR (Commercial Resort) Zone within the Airport Environs (AE-60) Overlay.</t>
   </si>
   <si>
-    <t>Clark County | approved</t>
+    <t>Clark County | filed</t>
   </si>
   <si>
     <t>Records show 5 filings and 3 press reports between 2026-05-26 and 2026-07-24.</t>
@@ -442,22 +445,16 @@
     <t>Party: Nancy Amundsen</t>
   </si>
   <si>
-    <t>representative; contact named in the record | Brown, Brown, &amp; Premsrirut | 520 S. 4th Street, Las Vegas, NV 89101 | No phone or email in the record.</t>
+    <t>representative; contact named in the filing | Brown, Brown, &amp; Premsrirut | 520 S. 4th Street, Las Vegas, NV 89101 | No phone or email in the record.</t>
   </si>
   <si>
     <t>Party: Eli Applebaum</t>
   </si>
   <si>
-    <t>https://www.mundovideo.com.co/en/america/ballys-chicago-and-skyvue-casino-plans-to-advance-in-illinois-and-nevada/</t>
-  </si>
-  <si>
-    <t>2026-05-26. Vacate and abandon easements of interest to Clark County located between Mandalay Bay Road and Four Seasons Drive, and Las Vegas Boulevard South and Haven Street; and a portion of a right-of-way being Mandalay Bay Road located between Las Vegas Boulevard South and Haven Street</t>
-  </si>
-  <si>
-    <t>VS-26-0218</t>
-  </si>
-  <si>
-    <t>https://www.clarkcountynv.gov/adobe/assets/urn:aaid:aem:bcdf1925-6c37-4308-b6f6-c718c78c9183/original/as/Paradise-Minutes-052626.pdf#item-vs-26-0218</t>
+    <t>named in press coverage | No phone or email in the record.</t>
+  </si>
+  <si>
+    <t>https://traveltomorrow.com/new-heart-shaped-hotel-approved-for-las-vegas-strip-sparks-debate-over-tacky-design/</t>
   </si>
   <si>
     <t>2026-05-26. Tentative map approval for 1 commercial lot on 11.95 acres in a CR (Commercial Resort) Zone within the Airport Environs (AE-60) Overlay</t>
@@ -466,6 +463,39 @@
     <t>TM-26-500056</t>
   </si>
   <si>
+    <t>2026-05-26. Use Permits to expand gaming enterprise district, construct resort hotel, and construct recreational facility; Waiver of Development Standards for non-standard improvements in right-of-way; Design Review for proposed resort hotel and recreational facility</t>
+  </si>
+  <si>
+    <t>UC-26-0219</t>
+  </si>
+  <si>
+    <t>https://www.clarkcountynv.gov/adobe/assets/urn:aaid:aem:bcdf1925-6c37-4308-b6f6-c718c78c9183/original/as/Paradise-Minutes-052626.pdf#item-uc-26-0219</t>
+  </si>
+  <si>
+    <t>2026-07-21. Holdover use permits to expand the gaming enterprise district, resort hotel, and recreational facility; Waiver of development standards to allow non-standard improvements in the right-of-way; Design review for a proposed resort hotel and recreational facility</t>
+  </si>
+  <si>
+    <t>UC-26-0219 | 11.95 acres | Contact: Nancy Amundsen, Brown, Brown, &amp; Premsrirut. No phone or email in the record.</t>
+  </si>
+  <si>
+    <t>https://clark.legistar.com/Legislation.aspx#matter-110426</t>
+  </si>
+  <si>
+    <t>2026-07-21. Vacate and abandon easements of interest to Clark County located between Mandalay Bay Road and Four Seasons Drive, and Las Vegas Boulevard South and Haven Street; and a portion of a right-of-way being Mandalay Bay Road located between Las Vegas Boulevard South and Haven Street within Paradise</t>
+  </si>
+  <si>
+    <t>VS-26-0218 | Contact: Nancy Amundsen, Brown, Brown, &amp; Premsrirut. No phone or email in the record.</t>
+  </si>
+  <si>
+    <t>https://clark.legistar.com/Legislation.aspx#matter-110425</t>
+  </si>
+  <si>
+    <t>2026-07-21. Resort project replacing failed Las Vegas Strip observation ...</t>
+  </si>
+  <si>
+    <t>https://news3lv.com/news/local/resort-project-skyvue-failed-las-vegas-strip-observation-wheel-clark-county-commission-zoning-approval</t>
+  </si>
+  <si>
     <t>2026-07-21. Holdover tentative map</t>
   </si>
   <si>
@@ -475,30 +505,6 @@
     <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110427</t>
   </si>
   <si>
-    <t>2026-07-21. Vacate and abandon easements of interest to Clark County located between Mandalay Bay Road and Four Seasons Drive, and Las Vegas Boulevard South and Haven Street; and a portion of a right-of-way being Mandalay Bay Road located between Las Vegas Boulevard South and Haven Street within Paradise</t>
-  </si>
-  <si>
-    <t>VS-26-0218 | Contact: Nancy Amundsen, Brown, Brown, &amp; Premsrirut. No phone or email in the record.</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/Legislation.aspx#matter-110425</t>
-  </si>
-  <si>
-    <t>2026-07-21. Resort project replacing failed Las Vegas Strip observation ...</t>
-  </si>
-  <si>
-    <t>https://news3lv.com/news/local/resort-project-skyvue-failed-las-vegas-strip-observation-wheel-clark-county-commission-zoning-approval</t>
-  </si>
-  <si>
-    <t>2026-07-21. Holdover use permits to expand the gaming enterprise district, resort hotel, and recreational facility; Waiver of development standards to allow non-standard improvements in the right-of-way; Design review for a proposed resort hotel and recreational facility</t>
-  </si>
-  <si>
-    <t>UC-26-0219 | 11.95 acres | Contact: Nancy Amundsen, Brown, Brown, &amp; Premsrirut. No phone or email in the record.</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/Legislation.aspx#matter-110426</t>
-  </si>
-  <si>
     <t>2026-07-23. Las Vegas Approves Heart-Shaped Casino on SkyVue Site</t>
   </si>
   <si>
@@ -523,7 +529,7 @@
     <t>Dormant projects are excluded from this report. None in this geography is dormant.</t>
   </si>
   <si>
-    <t>9 projects this scope proposes are held out of this document because they have not been confirmed as part of Simtec Attractions' coverage. A scope is a proposal: it finds projects that look like a match, and each one is confirmed by hand on the register before it may be printed. Those projects are on the register, unconfirmed, and are not a statement that they do not belong here. Confirming them on the register and regenerating is what puts them in this document.</t>
+    <t>40 projects this scope proposes are held out of this document because they have not been confirmed as part of Simtec Attractions' coverage. A scope is a proposal: it finds projects that look like a match, and each one is confirmed by hand on the register before it may be printed. Those projects are on the register, unconfirmed, and are not a statement that they do not belong here. Confirming them on the register and regenerating is what puts them in this document.</t>
   </si>
   <si>
     <t>This document describes the 15 most significant projects in scope. Every project in scope is described.</t>
@@ -919,7 +925,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1027,16 +1033,16 @@
         <v>13</v>
       </c>
       <c r="C11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" t="s">
         <v>21</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" t="s">
         <v>22</v>
-      </c>
-      <c r="E11" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1047,7 +1053,7 @@
         <v>13</v>
       </c>
       <c r="C12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D12" t="s">
         <v>24</v>
@@ -1067,7 +1073,7 @@
         <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D13" t="s">
         <v>27</v>
@@ -1087,7 +1093,7 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D14" t="s">
         <v>29</v>
@@ -1107,7 +1113,7 @@
         <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D15" t="s">
         <v>32</v>
@@ -1127,7 +1133,7 @@
         <v>13</v>
       </c>
       <c r="C16" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D16" t="s">
         <v>34</v>
@@ -1147,7 +1153,7 @@
         <v>13</v>
       </c>
       <c r="C17" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D17" t="s">
         <v>37</v>
@@ -1167,7 +1173,7 @@
         <v>13</v>
       </c>
       <c r="C18" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D18" t="s">
         <v>40</v>
@@ -1187,7 +1193,7 @@
         <v>42</v>
       </c>
       <c r="C19" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D19" t="s">
         <v>43</v>
@@ -1196,7 +1202,7 @@
         <v>44</v>
       </c>
       <c r="F19" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1227,7 +1233,7 @@
         <v>42</v>
       </c>
       <c r="C21" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D21" t="s">
         <v>46</v>
@@ -1236,7 +1242,7 @@
         <v>47</v>
       </c>
       <c r="F21" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1247,7 +1253,7 @@
         <v>42</v>
       </c>
       <c r="C22" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D22" t="s">
         <v>48</v>
@@ -1256,7 +1262,7 @@
         <v>47</v>
       </c>
       <c r="F22" t="s">
-        <v>26</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1267,16 +1273,16 @@
         <v>42</v>
       </c>
       <c r="C23" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E23" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F23" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1287,16 +1293,16 @@
         <v>42</v>
       </c>
       <c r="C24" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D24" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E24" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F24" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -1307,16 +1313,16 @@
         <v>42</v>
       </c>
       <c r="C25" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D25" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E25" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F25" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1327,16 +1333,16 @@
         <v>42</v>
       </c>
       <c r="C26" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D26" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E26" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F26" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1347,16 +1353,16 @@
         <v>42</v>
       </c>
       <c r="C27" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D27" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E27" t="s">
         <v>13</v>
       </c>
       <c r="F27" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1367,16 +1373,16 @@
         <v>42</v>
       </c>
       <c r="C28" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D28" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E28" t="s">
         <v>13</v>
       </c>
       <c r="F28" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1387,16 +1393,16 @@
         <v>42</v>
       </c>
       <c r="C29" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D29" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E29" t="s">
         <v>13</v>
       </c>
       <c r="F29" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -1407,16 +1413,16 @@
         <v>42</v>
       </c>
       <c r="C30" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D30" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E30" t="s">
         <v>13</v>
       </c>
       <c r="F30" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -1427,16 +1433,16 @@
         <v>42</v>
       </c>
       <c r="C31" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D31" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E31" t="s">
         <v>13</v>
       </c>
       <c r="F31" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1447,16 +1453,16 @@
         <v>42</v>
       </c>
       <c r="C32" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D32" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E32" t="s">
         <v>13</v>
       </c>
       <c r="F32" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1467,16 +1473,16 @@
         <v>42</v>
       </c>
       <c r="C33" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D33" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E33" t="s">
         <v>13</v>
       </c>
       <c r="F33" t="s">
-        <v>72</v>
+        <v>20</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1487,7 +1493,7 @@
         <v>73</v>
       </c>
       <c r="C34" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D34" t="s">
         <v>74</v>
@@ -1527,7 +1533,7 @@
         <v>73</v>
       </c>
       <c r="C36" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D36" t="s">
         <v>76</v>
@@ -1547,7 +1553,7 @@
         <v>73</v>
       </c>
       <c r="C37" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D37" t="s">
         <v>77</v>
@@ -1567,7 +1573,7 @@
         <v>73</v>
       </c>
       <c r="C38" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D38" t="s">
         <v>79</v>
@@ -1587,13 +1593,13 @@
         <v>73</v>
       </c>
       <c r="C39" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D39" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E39" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F39" t="s">
         <v>78</v>
@@ -1607,7 +1613,7 @@
         <v>73</v>
       </c>
       <c r="C40" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D40" t="s">
         <v>81</v>
@@ -1627,7 +1633,7 @@
         <v>73</v>
       </c>
       <c r="C41" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D41" t="s">
         <v>83</v>
@@ -1647,7 +1653,7 @@
         <v>73</v>
       </c>
       <c r="C42" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D42" t="s">
         <v>85</v>
@@ -1667,7 +1673,7 @@
         <v>73</v>
       </c>
       <c r="C43" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D43" t="s">
         <v>87</v>
@@ -1707,7 +1713,7 @@
         <v>88</v>
       </c>
       <c r="C45" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D45" t="s">
         <v>91</v>
@@ -1727,7 +1733,7 @@
         <v>88</v>
       </c>
       <c r="C46" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D46" t="s">
         <v>93</v>
@@ -1736,7 +1742,7 @@
         <v>94</v>
       </c>
       <c r="F46" t="s">
-        <v>36</v>
+        <v>92</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -1747,7 +1753,7 @@
         <v>88</v>
       </c>
       <c r="C47" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D47" t="s">
         <v>95</v>
@@ -1756,7 +1762,7 @@
         <v>96</v>
       </c>
       <c r="F47" t="s">
-        <v>92</v>
+        <v>36</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -1767,7 +1773,7 @@
         <v>88</v>
       </c>
       <c r="C48" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D48" t="s">
         <v>97</v>
@@ -1787,7 +1793,7 @@
         <v>88</v>
       </c>
       <c r="C49" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D49" t="s">
         <v>99</v>
@@ -1807,7 +1813,7 @@
         <v>88</v>
       </c>
       <c r="C50" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D50" t="s">
         <v>101</v>
@@ -1827,7 +1833,7 @@
         <v>104</v>
       </c>
       <c r="C51" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D51" t="s">
         <v>105</v>
@@ -1867,7 +1873,7 @@
         <v>104</v>
       </c>
       <c r="C53" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D53" t="s">
         <v>107</v>
@@ -1887,16 +1893,16 @@
         <v>104</v>
       </c>
       <c r="C54" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D54" t="s">
         <v>109</v>
       </c>
       <c r="E54" t="s">
+        <v>54</v>
+      </c>
+      <c r="F54" t="s">
         <v>110</v>
-      </c>
-      <c r="F54" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -1907,16 +1913,16 @@
         <v>104</v>
       </c>
       <c r="C55" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D55" t="s">
+        <v>111</v>
+      </c>
+      <c r="E55" t="s">
         <v>112</v>
       </c>
-      <c r="E55" t="s">
-        <v>113</v>
-      </c>
       <c r="F55" t="s">
-        <v>39</v>
+        <v>110</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -1927,16 +1933,16 @@
         <v>104</v>
       </c>
       <c r="C56" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D56" t="s">
+        <v>113</v>
+      </c>
+      <c r="E56" t="s">
         <v>114</v>
       </c>
-      <c r="E56" t="s">
-        <v>115</v>
-      </c>
       <c r="F56" t="s">
-        <v>116</v>
+        <v>39</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -1947,16 +1953,16 @@
         <v>104</v>
       </c>
       <c r="C57" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D57" t="s">
+        <v>115</v>
+      </c>
+      <c r="E57" t="s">
+        <v>116</v>
+      </c>
+      <c r="F57" t="s">
         <v>117</v>
-      </c>
-      <c r="E57" t="s">
-        <v>118</v>
-      </c>
-      <c r="F57" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -1967,16 +1973,16 @@
         <v>104</v>
       </c>
       <c r="C58" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D58" t="s">
+        <v>118</v>
+      </c>
+      <c r="E58" t="s">
+        <v>119</v>
+      </c>
+      <c r="F58" t="s">
         <v>120</v>
-      </c>
-      <c r="E58" t="s">
-        <v>121</v>
-      </c>
-      <c r="F58" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -1987,16 +1993,16 @@
         <v>104</v>
       </c>
       <c r="C59" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D59" t="s">
+        <v>121</v>
+      </c>
+      <c r="E59" t="s">
+        <v>122</v>
+      </c>
+      <c r="F59" t="s">
         <v>123</v>
-      </c>
-      <c r="E59" t="s">
-        <v>124</v>
-      </c>
-      <c r="F59" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -2007,16 +2013,16 @@
         <v>104</v>
       </c>
       <c r="C60" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D60" t="s">
+        <v>124</v>
+      </c>
+      <c r="E60" t="s">
+        <v>125</v>
+      </c>
+      <c r="F60" t="s">
         <v>126</v>
-      </c>
-      <c r="E60" t="s">
-        <v>127</v>
-      </c>
-      <c r="F60" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
@@ -2027,16 +2033,16 @@
         <v>104</v>
       </c>
       <c r="C61" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D61" t="s">
+        <v>127</v>
+      </c>
+      <c r="E61" t="s">
         <v>128</v>
       </c>
-      <c r="E61" t="s">
-        <v>13</v>
-      </c>
       <c r="F61" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
@@ -2047,16 +2053,16 @@
         <v>104</v>
       </c>
       <c r="C62" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D62" t="s">
+        <v>129</v>
+      </c>
+      <c r="E62" t="s">
+        <v>13</v>
+      </c>
+      <c r="F62" t="s">
         <v>130</v>
-      </c>
-      <c r="E62" t="s">
-        <v>131</v>
-      </c>
-      <c r="F62" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -2067,213 +2073,213 @@
         <v>104</v>
       </c>
       <c r="C63" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D63" t="s">
+        <v>131</v>
+      </c>
+      <c r="E63" t="s">
+        <v>132</v>
+      </c>
+      <c r="F63" t="s">
         <v>133</v>
-      </c>
-      <c r="E63" t="s">
-        <v>134</v>
-      </c>
-      <c r="F63" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>103</v>
+      </c>
+      <c r="B64" t="s">
+        <v>104</v>
+      </c>
+      <c r="C64" t="s">
+        <v>17</v>
+      </c>
+      <c r="D64" t="s">
+        <v>134</v>
+      </c>
+      <c r="E64" t="s">
         <v>135</v>
       </c>
-      <c r="B64" t="s">
-        <v>136</v>
-      </c>
-      <c r="C64" t="s">
-        <v>21</v>
-      </c>
-      <c r="D64" t="s">
-        <v>137</v>
-      </c>
-      <c r="E64" t="s">
-        <v>138</v>
-      </c>
       <c r="F64" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B65" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C65" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D65" t="s">
+        <v>138</v>
+      </c>
+      <c r="E65" t="s">
         <v>139</v>
       </c>
-      <c r="E65" t="s">
-        <v>138</v>
-      </c>
       <c r="F65" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B66" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C66" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D66" t="s">
         <v>140</v>
       </c>
       <c r="E66" t="s">
-        <v>47</v>
+        <v>139</v>
       </c>
       <c r="F66" t="s">
-        <v>141</v>
+        <v>13</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B67" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C67" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D67" t="s">
+        <v>141</v>
+      </c>
+      <c r="E67" t="s">
+        <v>47</v>
+      </c>
+      <c r="F67" t="s">
         <v>142</v>
-      </c>
-      <c r="E67" t="s">
-        <v>143</v>
-      </c>
-      <c r="F67" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B68" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C68" t="s">
         <v>17</v>
       </c>
       <c r="D68" t="s">
+        <v>143</v>
+      </c>
+      <c r="E68" t="s">
         <v>144</v>
       </c>
-      <c r="E68" t="s">
-        <v>113</v>
-      </c>
       <c r="F68" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B69" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C69" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D69" t="s">
+        <v>145</v>
+      </c>
+      <c r="E69" t="s">
         <v>146</v>
       </c>
-      <c r="E69" t="s">
+      <c r="F69" t="s">
         <v>147</v>
-      </c>
-      <c r="F69" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B70" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C70" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D70" t="s">
+        <v>148</v>
+      </c>
+      <c r="E70" t="s">
         <v>149</v>
       </c>
-      <c r="E70" t="s">
-        <v>150</v>
-      </c>
       <c r="F70" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B71" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C71" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D71" t="s">
+        <v>150</v>
+      </c>
+      <c r="E71" t="s">
         <v>151</v>
       </c>
-      <c r="E71" t="s">
+      <c r="F71" t="s">
         <v>152</v>
-      </c>
-      <c r="F71" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B72" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C72" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D72" t="s">
+        <v>153</v>
+      </c>
+      <c r="E72" t="s">
         <v>154</v>
       </c>
-      <c r="E72" t="s">
+      <c r="F72" t="s">
         <v>155</v>
-      </c>
-      <c r="F72" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B73" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C73" t="s">
         <v>17</v>
       </c>
       <c r="D73" t="s">
+        <v>156</v>
+      </c>
+      <c r="E73" t="s">
         <v>157</v>
-      </c>
-      <c r="E73" t="s">
-        <v>13</v>
       </c>
       <c r="F73" t="s">
         <v>158</v>
@@ -2281,39 +2287,39 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B74" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C74" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D74" t="s">
         <v>159</v>
       </c>
       <c r="E74" t="s">
+        <v>13</v>
+      </c>
+      <c r="F74" t="s">
         <v>160</v>
-      </c>
-      <c r="F74" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B75" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C75" t="s">
         <v>17</v>
       </c>
       <c r="D75" t="s">
+        <v>161</v>
+      </c>
+      <c r="E75" t="s">
         <v>162</v>
-      </c>
-      <c r="E75" t="s">
-        <v>13</v>
       </c>
       <c r="F75" t="s">
         <v>163</v>
@@ -2321,13 +2327,13 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B76" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C76" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D76" t="s">
         <v>164</v>
@@ -2336,72 +2342,72 @@
         <v>13</v>
       </c>
       <c r="F76" t="s">
-        <v>20</v>
+        <v>165</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>165</v>
+        <v>136</v>
       </c>
       <c r="B77" t="s">
-        <v>13</v>
+        <v>137</v>
       </c>
       <c r="C77" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D77" t="s">
-        <v>18</v>
+        <v>166</v>
       </c>
       <c r="E77" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F77" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B78" t="s">
         <v>13</v>
       </c>
       <c r="C78" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D78" t="s">
-        <v>167</v>
+        <v>18</v>
       </c>
       <c r="E78" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F78" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B79" t="s">
         <v>13</v>
       </c>
       <c r="C79" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D79" t="s">
-        <v>168</v>
+        <v>24</v>
       </c>
       <c r="E79" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F79" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B80" t="s">
         <v>13</v>
@@ -2421,7 +2427,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B81" t="s">
         <v>13</v>
@@ -2441,7 +2447,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B82" t="s">
         <v>13</v>
@@ -2461,7 +2467,7 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B83" t="s">
         <v>13</v>
@@ -2481,7 +2487,7 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B84" t="s">
         <v>13</v>
@@ -2501,7 +2507,7 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B85" t="s">
         <v>13</v>
@@ -2521,7 +2527,7 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B86" t="s">
         <v>13</v>
@@ -2536,6 +2542,46 @@
         <v>13</v>
       </c>
       <c r="F86" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>168</v>
+      </c>
+      <c r="B87" t="s">
+        <v>13</v>
+      </c>
+      <c r="C87" t="s">
+        <v>14</v>
+      </c>
+      <c r="D87" t="s">
+        <v>176</v>
+      </c>
+      <c r="E87" t="s">
+        <v>13</v>
+      </c>
+      <c r="F87" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>168</v>
+      </c>
+      <c r="B88" t="s">
+        <v>13</v>
+      </c>
+      <c r="C88" t="s">
+        <v>14</v>
+      </c>
+      <c r="D88" t="s">
+        <v>177</v>
+      </c>
+      <c r="E88" t="s">
+        <v>13</v>
+      </c>
+      <c r="F88" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
shots: regenerate from the green run after the brief blemishes
The referral brief is the artefact worth opening: a Matter row above the
Geography row, one citation on 51 conditions instead of 51, three press figures
on one line under one quotation, the LinkedIn post withheld with its count
stated, and the merged-record reconciliation printed once.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/e2e/shots/documents/full-report.xlsx
+++ b/dashboard/e2e/shots/documents/full-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="179">
   <si>
     <t>Market intelligence report</t>
   </si>
@@ -296,6 +296,9 @@
   </si>
   <si>
     <t>presented by | Director, Planning &amp; Engineering Department: Public Works | No phone or email in the record.</t>
+  </si>
+  <si>
+    <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/1-23-2026-BOS-Agenda-Packet-FINALcs.pdf#item-10-p4</t>
   </si>
   <si>
     <t>Party: Craig Sandt</t>
@@ -1742,7 +1745,7 @@
         <v>94</v>
       </c>
       <c r="F46" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -1756,10 +1759,10 @@
         <v>17</v>
       </c>
       <c r="D47" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E47" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F47" t="s">
         <v>36</v>
@@ -1776,13 +1779,13 @@
         <v>17</v>
       </c>
       <c r="D48" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E48" t="s">
         <v>13</v>
       </c>
       <c r="F48" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -1796,10 +1799,10 @@
         <v>17</v>
       </c>
       <c r="D49" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E49" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F49" t="s">
         <v>36</v>
@@ -1816,10 +1819,10 @@
         <v>17</v>
       </c>
       <c r="D50" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E50" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F50" t="s">
         <v>92</v>
@@ -1827,16 +1830,16 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B51" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C51" t="s">
         <v>17</v>
       </c>
       <c r="D51" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E51" t="s">
         <v>44</v>
@@ -1847,16 +1850,16 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B52" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C52" t="s">
         <v>13</v>
       </c>
       <c r="D52" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E52" t="s">
         <v>44</v>
@@ -1867,19 +1870,19 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B53" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C53" t="s">
         <v>17</v>
       </c>
       <c r="D53" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E53" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F53" t="s">
         <v>39</v>
@@ -1887,59 +1890,59 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B54" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C54" t="s">
         <v>17</v>
       </c>
       <c r="D54" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E54" t="s">
         <v>54</v>
       </c>
       <c r="F54" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B55" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C55" t="s">
         <v>17</v>
       </c>
       <c r="D55" t="s">
+        <v>112</v>
+      </c>
+      <c r="E55" t="s">
+        <v>113</v>
+      </c>
+      <c r="F55" t="s">
         <v>111</v>
-      </c>
-      <c r="E55" t="s">
-        <v>112</v>
-      </c>
-      <c r="F55" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B56" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C56" t="s">
         <v>17</v>
       </c>
       <c r="D56" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E56" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F56" t="s">
         <v>39</v>
@@ -1947,159 +1950,159 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B57" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C57" t="s">
         <v>17</v>
       </c>
       <c r="D57" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E57" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F57" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B58" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C58" t="s">
         <v>17</v>
       </c>
       <c r="D58" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E58" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F58" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B59" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C59" t="s">
         <v>17</v>
       </c>
       <c r="D59" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E59" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F59" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B60" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C60" t="s">
         <v>17</v>
       </c>
       <c r="D60" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E60" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F60" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B61" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C61" t="s">
         <v>17</v>
       </c>
       <c r="D61" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E61" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F61" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B62" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C62" t="s">
         <v>17</v>
       </c>
       <c r="D62" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E62" t="s">
         <v>13</v>
       </c>
       <c r="F62" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B63" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C63" t="s">
         <v>17</v>
       </c>
       <c r="D63" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E63" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F63" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B64" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C64" t="s">
         <v>17</v>
       </c>
       <c r="D64" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E64" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F64" t="s">
         <v>39</v>
@@ -2107,19 +2110,19 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B65" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C65" t="s">
         <v>17</v>
       </c>
       <c r="D65" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E65" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F65" t="s">
         <v>28</v>
@@ -2127,19 +2130,19 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B66" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C66" t="s">
         <v>13</v>
       </c>
       <c r="D66" t="s">
+        <v>141</v>
+      </c>
+      <c r="E66" t="s">
         <v>140</v>
-      </c>
-      <c r="E66" t="s">
-        <v>139</v>
       </c>
       <c r="F66" t="s">
         <v>13</v>
@@ -2147,79 +2150,79 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B67" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C67" t="s">
         <v>17</v>
       </c>
       <c r="D67" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E67" t="s">
         <v>47</v>
       </c>
       <c r="F67" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B68" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C68" t="s">
         <v>17</v>
       </c>
       <c r="D68" t="s">
+        <v>144</v>
+      </c>
+      <c r="E68" t="s">
+        <v>145</v>
+      </c>
+      <c r="F68" t="s">
         <v>143</v>
-      </c>
-      <c r="E68" t="s">
-        <v>144</v>
-      </c>
-      <c r="F68" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B69" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C69" t="s">
         <v>23</v>
       </c>
       <c r="D69" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E69" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F69" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B70" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C70" t="s">
         <v>17</v>
       </c>
       <c r="D70" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E70" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F70" t="s">
         <v>28</v>
@@ -2227,136 +2230,136 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B71" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C71" t="s">
         <v>17</v>
       </c>
       <c r="D71" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E71" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F71" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B72" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C72" t="s">
         <v>17</v>
       </c>
       <c r="D72" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E72" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F72" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B73" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C73" t="s">
         <v>17</v>
       </c>
       <c r="D73" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E73" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F73" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B74" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C74" t="s">
         <v>23</v>
       </c>
       <c r="D74" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E74" t="s">
         <v>13</v>
       </c>
       <c r="F74" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B75" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C75" t="s">
         <v>17</v>
       </c>
       <c r="D75" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E75" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F75" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B76" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C76" t="s">
         <v>23</v>
       </c>
       <c r="D76" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E76" t="s">
         <v>13</v>
       </c>
       <c r="F76" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B77" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C77" t="s">
         <v>23</v>
       </c>
       <c r="D77" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E77" t="s">
         <v>13</v>
@@ -2367,7 +2370,7 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B78" t="s">
         <v>13</v>
@@ -2387,7 +2390,7 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B79" t="s">
         <v>13</v>
@@ -2407,7 +2410,7 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B80" t="s">
         <v>13</v>
@@ -2416,7 +2419,7 @@
         <v>14</v>
       </c>
       <c r="D80" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E80" t="s">
         <v>13</v>
@@ -2427,7 +2430,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B81" t="s">
         <v>13</v>
@@ -2436,7 +2439,7 @@
         <v>14</v>
       </c>
       <c r="D81" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E81" t="s">
         <v>13</v>
@@ -2447,7 +2450,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B82" t="s">
         <v>13</v>
@@ -2456,7 +2459,7 @@
         <v>14</v>
       </c>
       <c r="D82" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E82" t="s">
         <v>13</v>
@@ -2467,7 +2470,7 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B83" t="s">
         <v>13</v>
@@ -2476,7 +2479,7 @@
         <v>14</v>
       </c>
       <c r="D83" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E83" t="s">
         <v>13</v>
@@ -2487,7 +2490,7 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B84" t="s">
         <v>13</v>
@@ -2496,7 +2499,7 @@
         <v>14</v>
       </c>
       <c r="D84" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E84" t="s">
         <v>13</v>
@@ -2507,7 +2510,7 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B85" t="s">
         <v>13</v>
@@ -2516,7 +2519,7 @@
         <v>14</v>
       </c>
       <c r="D85" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E85" t="s">
         <v>13</v>
@@ -2527,7 +2530,7 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B86" t="s">
         <v>13</v>
@@ -2536,7 +2539,7 @@
         <v>14</v>
       </c>
       <c r="D86" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E86" t="s">
         <v>13</v>
@@ -2547,7 +2550,7 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B87" t="s">
         <v>13</v>
@@ -2556,7 +2559,7 @@
         <v>14</v>
       </c>
       <c r="D87" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E87" t="s">
         <v>13</v>
@@ -2567,7 +2570,7 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B88" t="s">
         <v>13</v>
@@ -2576,7 +2579,7 @@
         <v>14</v>
       </c>
       <c r="D88" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E88" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
shots: regenerate from the 71 of 71 run with the stage reconciliation
The referral brief now carries the sentence migration 040 was run for: what our
filings support, what the press reports, and that the difference is our capture.
Its provenance tally moves from 77/21/5 to 77/18/6 - three fewer press lines from
the grouped figures, one more assessment from the withheld self-published post.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/e2e/shots/documents/full-report.xlsx
+++ b/dashboard/e2e/shots/documents/full-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="178">
   <si>
     <t>Market intelligence report</t>
   </si>
@@ -296,9 +296,6 @@
   </si>
   <si>
     <t>presented by | Director, Planning &amp; Engineering Department: Public Works | No phone or email in the record.</t>
-  </si>
-  <si>
-    <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/1-23-2026-BOS-Agenda-Packet-FINALcs.pdf#item-10-p4</t>
   </si>
   <si>
     <t>Party: Craig Sandt</t>
@@ -1745,7 +1742,7 @@
         <v>94</v>
       </c>
       <c r="F46" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -1759,10 +1756,10 @@
         <v>17</v>
       </c>
       <c r="D47" t="s">
+        <v>95</v>
+      </c>
+      <c r="E47" t="s">
         <v>96</v>
-      </c>
-      <c r="E47" t="s">
-        <v>97</v>
       </c>
       <c r="F47" t="s">
         <v>36</v>
@@ -1779,13 +1776,13 @@
         <v>17</v>
       </c>
       <c r="D48" t="s">
+        <v>97</v>
+      </c>
+      <c r="E48" t="s">
+        <v>13</v>
+      </c>
+      <c r="F48" t="s">
         <v>98</v>
-      </c>
-      <c r="E48" t="s">
-        <v>13</v>
-      </c>
-      <c r="F48" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -1799,10 +1796,10 @@
         <v>17</v>
       </c>
       <c r="D49" t="s">
+        <v>99</v>
+      </c>
+      <c r="E49" t="s">
         <v>100</v>
-      </c>
-      <c r="E49" t="s">
-        <v>101</v>
       </c>
       <c r="F49" t="s">
         <v>36</v>
@@ -1819,10 +1816,10 @@
         <v>17</v>
       </c>
       <c r="D50" t="s">
+        <v>101</v>
+      </c>
+      <c r="E50" t="s">
         <v>102</v>
-      </c>
-      <c r="E50" t="s">
-        <v>103</v>
       </c>
       <c r="F50" t="s">
         <v>92</v>
@@ -1830,16 +1827,16 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B51" t="s">
         <v>104</v>
       </c>
-      <c r="B51" t="s">
+      <c r="C51" t="s">
+        <v>17</v>
+      </c>
+      <c r="D51" t="s">
         <v>105</v>
-      </c>
-      <c r="C51" t="s">
-        <v>17</v>
-      </c>
-      <c r="D51" t="s">
-        <v>106</v>
       </c>
       <c r="E51" t="s">
         <v>44</v>
@@ -1850,16 +1847,16 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>103</v>
+      </c>
+      <c r="B52" t="s">
         <v>104</v>
       </c>
-      <c r="B52" t="s">
-        <v>105</v>
-      </c>
       <c r="C52" t="s">
         <v>13</v>
       </c>
       <c r="D52" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E52" t="s">
         <v>44</v>
@@ -1870,19 +1867,19 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>103</v>
+      </c>
+      <c r="B53" t="s">
         <v>104</v>
       </c>
-      <c r="B53" t="s">
-        <v>105</v>
-      </c>
       <c r="C53" t="s">
         <v>17</v>
       </c>
       <c r="D53" t="s">
+        <v>107</v>
+      </c>
+      <c r="E53" t="s">
         <v>108</v>
-      </c>
-      <c r="E53" t="s">
-        <v>109</v>
       </c>
       <c r="F53" t="s">
         <v>39</v>
@@ -1890,59 +1887,59 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>103</v>
+      </c>
+      <c r="B54" t="s">
         <v>104</v>
       </c>
-      <c r="B54" t="s">
-        <v>105</v>
-      </c>
       <c r="C54" t="s">
         <v>17</v>
       </c>
       <c r="D54" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E54" t="s">
         <v>54</v>
       </c>
       <c r="F54" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>103</v>
+      </c>
+      <c r="B55" t="s">
         <v>104</v>
       </c>
-      <c r="B55" t="s">
-        <v>105</v>
-      </c>
       <c r="C55" t="s">
         <v>17</v>
       </c>
       <c r="D55" t="s">
+        <v>111</v>
+      </c>
+      <c r="E55" t="s">
         <v>112</v>
       </c>
-      <c r="E55" t="s">
-        <v>113</v>
-      </c>
       <c r="F55" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>103</v>
+      </c>
+      <c r="B56" t="s">
         <v>104</v>
       </c>
-      <c r="B56" t="s">
-        <v>105</v>
-      </c>
       <c r="C56" t="s">
         <v>17</v>
       </c>
       <c r="D56" t="s">
+        <v>113</v>
+      </c>
+      <c r="E56" t="s">
         <v>114</v>
-      </c>
-      <c r="E56" t="s">
-        <v>115</v>
       </c>
       <c r="F56" t="s">
         <v>39</v>
@@ -1950,159 +1947,159 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>103</v>
+      </c>
+      <c r="B57" t="s">
         <v>104</v>
       </c>
-      <c r="B57" t="s">
-        <v>105</v>
-      </c>
       <c r="C57" t="s">
         <v>17</v>
       </c>
       <c r="D57" t="s">
+        <v>115</v>
+      </c>
+      <c r="E57" t="s">
         <v>116</v>
       </c>
-      <c r="E57" t="s">
+      <c r="F57" t="s">
         <v>117</v>
-      </c>
-      <c r="F57" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>103</v>
+      </c>
+      <c r="B58" t="s">
         <v>104</v>
       </c>
-      <c r="B58" t="s">
-        <v>105</v>
-      </c>
       <c r="C58" t="s">
         <v>17</v>
       </c>
       <c r="D58" t="s">
+        <v>118</v>
+      </c>
+      <c r="E58" t="s">
         <v>119</v>
       </c>
-      <c r="E58" t="s">
+      <c r="F58" t="s">
         <v>120</v>
-      </c>
-      <c r="F58" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>103</v>
+      </c>
+      <c r="B59" t="s">
         <v>104</v>
       </c>
-      <c r="B59" t="s">
-        <v>105</v>
-      </c>
       <c r="C59" t="s">
         <v>17</v>
       </c>
       <c r="D59" t="s">
+        <v>121</v>
+      </c>
+      <c r="E59" t="s">
         <v>122</v>
       </c>
-      <c r="E59" t="s">
+      <c r="F59" t="s">
         <v>123</v>
-      </c>
-      <c r="F59" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>103</v>
+      </c>
+      <c r="B60" t="s">
         <v>104</v>
       </c>
-      <c r="B60" t="s">
-        <v>105</v>
-      </c>
       <c r="C60" t="s">
         <v>17</v>
       </c>
       <c r="D60" t="s">
+        <v>124</v>
+      </c>
+      <c r="E60" t="s">
         <v>125</v>
       </c>
-      <c r="E60" t="s">
+      <c r="F60" t="s">
         <v>126</v>
-      </c>
-      <c r="F60" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>103</v>
+      </c>
+      <c r="B61" t="s">
         <v>104</v>
       </c>
-      <c r="B61" t="s">
-        <v>105</v>
-      </c>
       <c r="C61" t="s">
         <v>17</v>
       </c>
       <c r="D61" t="s">
+        <v>127</v>
+      </c>
+      <c r="E61" t="s">
         <v>128</v>
       </c>
-      <c r="E61" t="s">
-        <v>129</v>
-      </c>
       <c r="F61" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>103</v>
+      </c>
+      <c r="B62" t="s">
         <v>104</v>
       </c>
-      <c r="B62" t="s">
-        <v>105</v>
-      </c>
       <c r="C62" t="s">
         <v>17</v>
       </c>
       <c r="D62" t="s">
+        <v>129</v>
+      </c>
+      <c r="E62" t="s">
+        <v>13</v>
+      </c>
+      <c r="F62" t="s">
         <v>130</v>
-      </c>
-      <c r="E62" t="s">
-        <v>13</v>
-      </c>
-      <c r="F62" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>103</v>
+      </c>
+      <c r="B63" t="s">
         <v>104</v>
       </c>
-      <c r="B63" t="s">
-        <v>105</v>
-      </c>
       <c r="C63" t="s">
         <v>17</v>
       </c>
       <c r="D63" t="s">
+        <v>131</v>
+      </c>
+      <c r="E63" t="s">
         <v>132</v>
       </c>
-      <c r="E63" t="s">
+      <c r="F63" t="s">
         <v>133</v>
-      </c>
-      <c r="F63" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>103</v>
+      </c>
+      <c r="B64" t="s">
         <v>104</v>
       </c>
-      <c r="B64" t="s">
-        <v>105</v>
-      </c>
       <c r="C64" t="s">
         <v>17</v>
       </c>
       <c r="D64" t="s">
+        <v>134</v>
+      </c>
+      <c r="E64" t="s">
         <v>135</v>
-      </c>
-      <c r="E64" t="s">
-        <v>136</v>
       </c>
       <c r="F64" t="s">
         <v>39</v>
@@ -2110,19 +2107,19 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>136</v>
+      </c>
+      <c r="B65" t="s">
         <v>137</v>
       </c>
-      <c r="B65" t="s">
+      <c r="C65" t="s">
+        <v>17</v>
+      </c>
+      <c r="D65" t="s">
         <v>138</v>
       </c>
-      <c r="C65" t="s">
-        <v>17</v>
-      </c>
-      <c r="D65" t="s">
+      <c r="E65" t="s">
         <v>139</v>
-      </c>
-      <c r="E65" t="s">
-        <v>140</v>
       </c>
       <c r="F65" t="s">
         <v>28</v>
@@ -2130,19 +2127,19 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>136</v>
+      </c>
+      <c r="B66" t="s">
         <v>137</v>
       </c>
-      <c r="B66" t="s">
-        <v>138</v>
-      </c>
       <c r="C66" t="s">
         <v>13</v>
       </c>
       <c r="D66" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E66" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F66" t="s">
         <v>13</v>
@@ -2150,79 +2147,79 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>136</v>
+      </c>
+      <c r="B67" t="s">
         <v>137</v>
       </c>
-      <c r="B67" t="s">
-        <v>138</v>
-      </c>
       <c r="C67" t="s">
         <v>17</v>
       </c>
       <c r="D67" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E67" t="s">
         <v>47</v>
       </c>
       <c r="F67" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>136</v>
+      </c>
+      <c r="B68" t="s">
         <v>137</v>
       </c>
-      <c r="B68" t="s">
-        <v>138</v>
-      </c>
       <c r="C68" t="s">
         <v>17</v>
       </c>
       <c r="D68" t="s">
+        <v>143</v>
+      </c>
+      <c r="E68" t="s">
         <v>144</v>
       </c>
-      <c r="E68" t="s">
-        <v>145</v>
-      </c>
       <c r="F68" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>136</v>
+      </c>
+      <c r="B69" t="s">
         <v>137</v>
-      </c>
-      <c r="B69" t="s">
-        <v>138</v>
       </c>
       <c r="C69" t="s">
         <v>23</v>
       </c>
       <c r="D69" t="s">
+        <v>145</v>
+      </c>
+      <c r="E69" t="s">
         <v>146</v>
       </c>
-      <c r="E69" t="s">
+      <c r="F69" t="s">
         <v>147</v>
-      </c>
-      <c r="F69" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>136</v>
+      </c>
+      <c r="B70" t="s">
         <v>137</v>
       </c>
-      <c r="B70" t="s">
-        <v>138</v>
-      </c>
       <c r="C70" t="s">
         <v>17</v>
       </c>
       <c r="D70" t="s">
+        <v>148</v>
+      </c>
+      <c r="E70" t="s">
         <v>149</v>
-      </c>
-      <c r="E70" t="s">
-        <v>150</v>
       </c>
       <c r="F70" t="s">
         <v>28</v>
@@ -2230,136 +2227,136 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>136</v>
+      </c>
+      <c r="B71" t="s">
         <v>137</v>
       </c>
-      <c r="B71" t="s">
-        <v>138</v>
-      </c>
       <c r="C71" t="s">
         <v>17</v>
       </c>
       <c r="D71" t="s">
+        <v>150</v>
+      </c>
+      <c r="E71" t="s">
         <v>151</v>
       </c>
-      <c r="E71" t="s">
+      <c r="F71" t="s">
         <v>152</v>
-      </c>
-      <c r="F71" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>136</v>
+      </c>
+      <c r="B72" t="s">
         <v>137</v>
       </c>
-      <c r="B72" t="s">
-        <v>138</v>
-      </c>
       <c r="C72" t="s">
         <v>17</v>
       </c>
       <c r="D72" t="s">
+        <v>153</v>
+      </c>
+      <c r="E72" t="s">
         <v>154</v>
       </c>
-      <c r="E72" t="s">
+      <c r="F72" t="s">
         <v>155</v>
-      </c>
-      <c r="F72" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>136</v>
+      </c>
+      <c r="B73" t="s">
         <v>137</v>
       </c>
-      <c r="B73" t="s">
-        <v>138</v>
-      </c>
       <c r="C73" t="s">
         <v>17</v>
       </c>
       <c r="D73" t="s">
+        <v>156</v>
+      </c>
+      <c r="E73" t="s">
         <v>157</v>
       </c>
-      <c r="E73" t="s">
+      <c r="F73" t="s">
         <v>158</v>
-      </c>
-      <c r="F73" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
+        <v>136</v>
+      </c>
+      <c r="B74" t="s">
         <v>137</v>
-      </c>
-      <c r="B74" t="s">
-        <v>138</v>
       </c>
       <c r="C74" t="s">
         <v>23</v>
       </c>
       <c r="D74" t="s">
+        <v>159</v>
+      </c>
+      <c r="E74" t="s">
+        <v>13</v>
+      </c>
+      <c r="F74" t="s">
         <v>160</v>
-      </c>
-      <c r="E74" t="s">
-        <v>13</v>
-      </c>
-      <c r="F74" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>136</v>
+      </c>
+      <c r="B75" t="s">
         <v>137</v>
       </c>
-      <c r="B75" t="s">
-        <v>138</v>
-      </c>
       <c r="C75" t="s">
         <v>17</v>
       </c>
       <c r="D75" t="s">
+        <v>161</v>
+      </c>
+      <c r="E75" t="s">
         <v>162</v>
       </c>
-      <c r="E75" t="s">
+      <c r="F75" t="s">
         <v>163</v>
-      </c>
-      <c r="F75" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>136</v>
+      </c>
+      <c r="B76" t="s">
         <v>137</v>
-      </c>
-      <c r="B76" t="s">
-        <v>138</v>
       </c>
       <c r="C76" t="s">
         <v>23</v>
       </c>
       <c r="D76" t="s">
+        <v>164</v>
+      </c>
+      <c r="E76" t="s">
+        <v>13</v>
+      </c>
+      <c r="F76" t="s">
         <v>165</v>
-      </c>
-      <c r="E76" t="s">
-        <v>13</v>
-      </c>
-      <c r="F76" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>136</v>
+      </c>
+      <c r="B77" t="s">
         <v>137</v>
-      </c>
-      <c r="B77" t="s">
-        <v>138</v>
       </c>
       <c r="C77" t="s">
         <v>23</v>
       </c>
       <c r="D77" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E77" t="s">
         <v>13</v>
@@ -2370,7 +2367,7 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B78" t="s">
         <v>13</v>
@@ -2390,7 +2387,7 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B79" t="s">
         <v>13</v>
@@ -2410,7 +2407,7 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B80" t="s">
         <v>13</v>
@@ -2419,7 +2416,7 @@
         <v>14</v>
       </c>
       <c r="D80" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E80" t="s">
         <v>13</v>
@@ -2430,7 +2427,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B81" t="s">
         <v>13</v>
@@ -2439,7 +2436,7 @@
         <v>14</v>
       </c>
       <c r="D81" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E81" t="s">
         <v>13</v>
@@ -2450,7 +2447,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B82" t="s">
         <v>13</v>
@@ -2459,7 +2456,7 @@
         <v>14</v>
       </c>
       <c r="D82" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E82" t="s">
         <v>13</v>
@@ -2470,7 +2467,7 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B83" t="s">
         <v>13</v>
@@ -2479,7 +2476,7 @@
         <v>14</v>
       </c>
       <c r="D83" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E83" t="s">
         <v>13</v>
@@ -2490,7 +2487,7 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B84" t="s">
         <v>13</v>
@@ -2499,7 +2496,7 @@
         <v>14</v>
       </c>
       <c r="D84" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E84" t="s">
         <v>13</v>
@@ -2510,7 +2507,7 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B85" t="s">
         <v>13</v>
@@ -2519,7 +2516,7 @@
         <v>14</v>
       </c>
       <c r="D85" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E85" t="s">
         <v>13</v>
@@ -2530,7 +2527,7 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B86" t="s">
         <v>13</v>
@@ -2539,7 +2536,7 @@
         <v>14</v>
       </c>
       <c r="D86" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E86" t="s">
         <v>13</v>
@@ -2550,7 +2547,7 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B87" t="s">
         <v>13</v>
@@ -2559,7 +2556,7 @@
         <v>14</v>
       </c>
       <c r="D87" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E87" t="s">
         <v>13</v>
@@ -2570,7 +2567,7 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B88" t="s">
         <v>13</v>
@@ -2579,7 +2576,7 @@
         <v>14</v>
       </c>
       <c r="D88" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E88" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
shots: regenerate from the 71 of 71 run with the presenter gate
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/e2e/shots/documents/full-report.xlsx
+++ b/dashboard/e2e/shots/documents/full-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="172">
   <si>
     <t>Market intelligence report</t>
   </si>
@@ -166,36 +166,30 @@
     <t>Party: Lisandro Orozco</t>
   </si>
   <si>
-    <t>presented by; contact named in the filing | lorozco@anaheim.net</t>
+    <t>contact named in the filing | lorozco@anaheim.net</t>
   </si>
   <si>
     <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_45b322ae69423ed7f4d96ffe8e8de725.pdf&amp;view=1#item-h9fe8d90cfc0b</t>
   </si>
   <si>
-    <t>Party: City of Anaheim</t>
-  </si>
-  <si>
-    <t>presented by | No phone or email in the record.</t>
+    <t>Party: Stacy Tran</t>
+  </si>
+  <si>
+    <t>contact named in the filing | STran@anaheim.net</t>
+  </si>
+  <si>
+    <t>https://www.anaheim.net/DocumentCenter/View/66931/Planning-Commission-Action-Agenda---10202025#item-h6dc7e70418cc</t>
+  </si>
+  <si>
+    <t>6 further records name the body that brought this matter forward (City of Anaheim; Lisandro Orozco; Stacy Tran). That is who moved it in government rather than who is behind it, so it is not listed above as a party to approach.</t>
+  </si>
+  <si>
+    <t>2026-02-06. OCVibe Residential Phase I</t>
   </si>
   <si>
     <t>https://ceqanet.lci.ca.gov/Project/2004121045</t>
   </si>
   <si>
-    <t>Party: Stacy Tran</t>
-  </si>
-  <si>
-    <t>presented by; contact named in the filing | STran@anaheim.net</t>
-  </si>
-  <si>
-    <t>https://www.anaheim.net/DocumentCenter/View/66931/Planning-Commission-Action-Agenda---10202025#item-h6dc7e70418cc</t>
-  </si>
-  <si>
-    <t>2026-02-06. OCVibe Residential Phase I</t>
-  </si>
-  <si>
-    <t>Players: City of Anaheim (presented by)</t>
-  </si>
-  <si>
     <t>2026-04-20. Approve Amendment No. 2 to Bond Purchase Agreement between the City of Anaheim, the Public Financing Authority, and JP Morgan amending the scheduled completion date to no later than June 25, 2027 for the parking decks associated with the OCVibe Project; and authorize the Finance Director to execute the amendment</t>
   </si>
   <si>
@@ -256,10 +250,13 @@
     <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_5713ee926e19136cdccede9cc8a3ce47.pdf&amp;view=1#item-h72954c9ae56e</t>
   </si>
   <si>
+    <t>One further record names the body that brought this matter forward (City of Anaheim). That is who moved it in government rather than who is behind it, so it is not listed above as a party to approach.</t>
+  </si>
+  <si>
     <t>2024-05-08. DisneylandForward Project</t>
   </si>
   <si>
-    <t>Players: Disneyland (applicant); City of Anaheim (presented by)</t>
+    <t>Players: Disneyland (applicant)</t>
   </si>
   <si>
     <t>2025-06-16. Determine compliance in good faith with terms and conditions of First Amended and Restated Development Agreement No. 96-01 for the 2024-2025 review period</t>
@@ -292,16 +289,7 @@
     <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/1-23-2026-BOS-Agenda-Packet-FINALcs.pdf#item-6.4-p146</t>
   </si>
   <si>
-    <t>Party: Katherine Luetzow</t>
-  </si>
-  <si>
-    <t>presented by | Director, Planning &amp; Engineering Department: Public Works | No phone or email in the record.</t>
-  </si>
-  <si>
-    <t>Party: Craig Sandt</t>
-  </si>
-  <si>
-    <t>presented by | Director of Construction Management | No phone or email in the record.</t>
+    <t>4 further records name the body that brought this matter forward (Craig Sandt, Director of Construction Management; Katherine Luetzow, Director, Planning &amp; Engineering Department: Public Works). That is who moved it in government rather than who is behind it, so it is not listed above as a party to approach.</t>
   </si>
   <si>
     <t>2026-01-01. CFTOD 2045 Comprehensive Plan - recreation / tourist provisions (p.37)</t>
@@ -313,15 +301,9 @@
     <t>2026-01-23. Approve the First Amendment to Roadway Expansion Land Dedication and Reimbursement Agreement and authorize the District Administrator or her designee to execute same</t>
   </si>
   <si>
-    <t>Players: Craig Sandt, Director of Construction Management (presented by)</t>
-  </si>
-  <si>
     <t>2026-01-23. Approve the District Administrator to execute a Non-exclusive temporary easement with permanent easement for underground communication lines</t>
   </si>
   <si>
-    <t>Players: Katherine Luetzow, Director, Planning &amp; Engineering Department: Public Works (presented by)</t>
-  </si>
-  <si>
     <t>Mixed-Use/Real Estate</t>
   </si>
   <si>
@@ -340,24 +322,24 @@
     <t>applicant | LLC and Joey Caucas | No phone or email in the record.</t>
   </si>
   <si>
-    <t>Party: City of Anaheim Planning Staff</t>
+    <t>Party: Christine Nguyen</t>
+  </si>
+  <si>
+    <t>contact named in the filing | CNguyen2@anaheim.net | Also presenter on 2 other projects in our register: 2 in Anaheim.</t>
   </si>
   <si>
     <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_2bfcbb0f5f83e7b944ef537de2b1fd4a.pdf&amp;view=1#item-ha13a91a5c59d</t>
   </si>
   <si>
-    <t>Party: Christine Nguyen</t>
-  </si>
-  <si>
-    <t>contact named in the filing | CNguyen2@anaheim.net | Also presenter on 2 other projects in our register: 2 in Anaheim.</t>
-  </si>
-  <si>
     <t>Party: Joey Caucas</t>
   </si>
   <si>
     <t>contact named in the filing | No phone or email in the record.</t>
   </si>
   <si>
+    <t>One further record names the body that brought this matter forward (City of Anaheim Planning Staff). That is who moved it in government rather than who is behind it, so it is not listed above as a party to approach.</t>
+  </si>
+  <si>
     <t>2025-01-13. Adoption of Ordinance No. 6601 amending multiple chapters of Title 18 (Zoning) of the Anaheim Municipal Code and adjustments to multiple specific plans</t>
   </si>
   <si>
@@ -397,7 +379,7 @@
     <t>2025-08-10. General Plan Amendment and Zoning Code amendments related to implementation of the Sixth Cycle Housing Element, including updates to General Plan Land Use Element Table LU-2 and amendments to Title 18 (Zoning) of the Anaheim Municipal Code</t>
   </si>
   <si>
-    <t>DEVELOPMENT APPLICATION No. 2021-00223 | Players: City of Anaheim Planning Staff (presented by) | Contact: Christine Nguyen. CNguyen2@anaheim.net.</t>
+    <t>DEVELOPMENT APPLICATION No. 2021-00223 | Contact: Christine Nguyen. CNguyen2@anaheim.net.</t>
   </si>
   <si>
     <t>2025-08-11. Levying Special Taxes within City of Anaheim Community Facilities District No. 06-2 (Stadium Lofts) and Community Facilities District No. 08-1 (Platinum Triangle)</t>
@@ -925,7 +907,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1313,16 +1295,16 @@
         <v>42</v>
       </c>
       <c r="C25" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D25" t="s">
         <v>56</v>
       </c>
       <c r="E25" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="F25" t="s">
-        <v>58</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1336,13 +1318,13 @@
         <v>17</v>
       </c>
       <c r="D26" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E26" t="s">
-        <v>60</v>
+        <v>13</v>
       </c>
       <c r="F26" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1356,13 +1338,13 @@
         <v>17</v>
       </c>
       <c r="D27" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E27" t="s">
         <v>13</v>
       </c>
       <c r="F27" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1376,13 +1358,13 @@
         <v>23</v>
       </c>
       <c r="D28" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E28" t="s">
         <v>13</v>
       </c>
       <c r="F28" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1396,7 +1378,7 @@
         <v>17</v>
       </c>
       <c r="D29" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E29" t="s">
         <v>13</v>
@@ -1416,13 +1398,13 @@
         <v>23</v>
       </c>
       <c r="D30" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E30" t="s">
         <v>13</v>
       </c>
       <c r="F30" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -1436,13 +1418,13 @@
         <v>23</v>
       </c>
       <c r="D31" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E31" t="s">
         <v>13</v>
       </c>
       <c r="F31" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1456,13 +1438,13 @@
         <v>23</v>
       </c>
       <c r="D32" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E32" t="s">
         <v>13</v>
       </c>
       <c r="F32" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1476,7 +1458,7 @@
         <v>17</v>
       </c>
       <c r="D33" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E33" t="s">
         <v>13</v>
@@ -1490,13 +1472,13 @@
         <v>41</v>
       </c>
       <c r="B34" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C34" t="s">
         <v>17</v>
       </c>
       <c r="D34" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E34" t="s">
         <v>44</v>
@@ -1510,13 +1492,13 @@
         <v>41</v>
       </c>
       <c r="B35" t="s">
+        <v>71</v>
+      </c>
+      <c r="C35" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" t="s">
         <v>73</v>
-      </c>
-      <c r="C35" t="s">
-        <v>13</v>
-      </c>
-      <c r="D35" t="s">
-        <v>75</v>
       </c>
       <c r="E35" t="s">
         <v>44</v>
@@ -1530,13 +1512,13 @@
         <v>41</v>
       </c>
       <c r="B36" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C36" t="s">
         <v>17</v>
       </c>
       <c r="D36" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E36" t="s">
         <v>47</v>
@@ -1550,19 +1532,19 @@
         <v>41</v>
       </c>
       <c r="B37" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C37" t="s">
         <v>17</v>
       </c>
       <c r="D37" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E37" t="s">
         <v>47</v>
       </c>
       <c r="F37" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -1570,19 +1552,19 @@
         <v>41</v>
       </c>
       <c r="B38" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C38" t="s">
         <v>17</v>
       </c>
       <c r="D38" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E38" t="s">
         <v>47</v>
       </c>
       <c r="F38" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -1590,19 +1572,19 @@
         <v>41</v>
       </c>
       <c r="B39" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C39" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D39" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="E39" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="F39" t="s">
-        <v>78</v>
+        <v>13</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -1610,19 +1592,19 @@
         <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C40" t="s">
         <v>17</v>
       </c>
       <c r="D40" t="s">
+        <v>80</v>
+      </c>
+      <c r="E40" t="s">
         <v>81</v>
       </c>
-      <c r="E40" t="s">
-        <v>82</v>
-      </c>
       <c r="F40" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -1630,19 +1612,19 @@
         <v>41</v>
       </c>
       <c r="B41" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C41" t="s">
         <v>17</v>
       </c>
       <c r="D41" t="s">
+        <v>82</v>
+      </c>
+      <c r="E41" t="s">
+        <v>13</v>
+      </c>
+      <c r="F41" t="s">
         <v>83</v>
-      </c>
-      <c r="E41" t="s">
-        <v>13</v>
-      </c>
-      <c r="F41" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -1650,16 +1632,16 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C42" t="s">
         <v>17</v>
       </c>
       <c r="D42" t="s">
+        <v>84</v>
+      </c>
+      <c r="E42" t="s">
         <v>85</v>
-      </c>
-      <c r="E42" t="s">
-        <v>86</v>
       </c>
       <c r="F42" t="s">
         <v>33</v>
@@ -1670,13 +1652,13 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C43" t="s">
         <v>17</v>
       </c>
       <c r="D43" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E43" t="s">
         <v>13</v>
@@ -1690,16 +1672,16 @@
         <v>41</v>
       </c>
       <c r="B44" t="s">
+        <v>87</v>
+      </c>
+      <c r="C44" t="s">
+        <v>13</v>
+      </c>
+      <c r="D44" t="s">
         <v>88</v>
       </c>
-      <c r="C44" t="s">
-        <v>13</v>
-      </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>89</v>
-      </c>
-      <c r="E44" t="s">
-        <v>90</v>
       </c>
       <c r="F44" t="s">
         <v>13</v>
@@ -1710,19 +1692,19 @@
         <v>41</v>
       </c>
       <c r="B45" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C45" t="s">
         <v>17</v>
       </c>
       <c r="D45" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E45" t="s">
         <v>47</v>
       </c>
       <c r="F45" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -1730,19 +1712,19 @@
         <v>41</v>
       </c>
       <c r="B46" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C46" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D46" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E46" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="F46" t="s">
-        <v>92</v>
+        <v>13</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -1750,19 +1732,19 @@
         <v>41</v>
       </c>
       <c r="B47" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C47" t="s">
         <v>17</v>
       </c>
       <c r="D47" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E47" t="s">
-        <v>96</v>
+        <v>13</v>
       </c>
       <c r="F47" t="s">
-        <v>36</v>
+        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -1770,19 +1752,19 @@
         <v>41</v>
       </c>
       <c r="B48" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C48" t="s">
         <v>17</v>
       </c>
       <c r="D48" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E48" t="s">
         <v>13</v>
       </c>
       <c r="F48" t="s">
-        <v>98</v>
+        <v>36</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -1790,624 +1772,624 @@
         <v>41</v>
       </c>
       <c r="B49" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C49" t="s">
         <v>17</v>
       </c>
       <c r="D49" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E49" t="s">
-        <v>100</v>
+        <v>13</v>
       </c>
       <c r="F49" t="s">
-        <v>36</v>
+        <v>91</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>41</v>
+        <v>97</v>
       </c>
       <c r="B50" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="C50" t="s">
         <v>17</v>
       </c>
       <c r="D50" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E50" t="s">
-        <v>102</v>
+        <v>44</v>
       </c>
       <c r="F50" t="s">
-        <v>92</v>
+        <v>39</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B51" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C51" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D51" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="E51" t="s">
         <v>44</v>
       </c>
       <c r="F51" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B52" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C52" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D52" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="E52" t="s">
-        <v>44</v>
+        <v>102</v>
       </c>
       <c r="F52" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>97</v>
+      </c>
+      <c r="B53" t="s">
+        <v>98</v>
+      </c>
+      <c r="C53" t="s">
+        <v>17</v>
+      </c>
+      <c r="D53" t="s">
         <v>103</v>
       </c>
-      <c r="B53" t="s">
+      <c r="E53" t="s">
         <v>104</v>
       </c>
-      <c r="C53" t="s">
-        <v>17</v>
-      </c>
-      <c r="D53" t="s">
-        <v>107</v>
-      </c>
-      <c r="E53" t="s">
-        <v>108</v>
-      </c>
       <c r="F53" t="s">
-        <v>39</v>
+        <v>105</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B54" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C54" t="s">
         <v>17</v>
       </c>
       <c r="D54" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E54" t="s">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="F54" t="s">
-        <v>110</v>
+        <v>39</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B55" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C55" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D55" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E55" t="s">
-        <v>112</v>
+        <v>44</v>
       </c>
       <c r="F55" t="s">
-        <v>110</v>
+        <v>13</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B56" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C56" t="s">
         <v>17</v>
       </c>
       <c r="D56" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="E56" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F56" t="s">
-        <v>39</v>
+        <v>111</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B57" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C57" t="s">
         <v>17</v>
       </c>
       <c r="D57" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E57" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F57" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B58" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C58" t="s">
         <v>17</v>
       </c>
       <c r="D58" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="E58" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="F58" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B59" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C59" t="s">
         <v>17</v>
       </c>
       <c r="D59" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E59" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F59" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B60" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C60" t="s">
         <v>17</v>
       </c>
       <c r="D60" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E60" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F60" t="s">
-        <v>126</v>
+        <v>105</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B61" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C61" t="s">
         <v>17</v>
       </c>
       <c r="D61" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E61" t="s">
-        <v>128</v>
+        <v>13</v>
       </c>
       <c r="F61" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B62" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C62" t="s">
         <v>17</v>
       </c>
       <c r="D62" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E62" t="s">
-        <v>13</v>
+        <v>126</v>
       </c>
       <c r="F62" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B63" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C63" t="s">
         <v>17</v>
       </c>
       <c r="D63" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E63" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F63" t="s">
-        <v>133</v>
+        <v>39</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="B64" t="s">
-        <v>104</v>
+        <v>131</v>
       </c>
       <c r="C64" t="s">
         <v>17</v>
       </c>
       <c r="D64" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E64" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F64" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B65" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C65" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D65" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E65" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="F65" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>130</v>
+      </c>
+      <c r="B66" t="s">
+        <v>131</v>
+      </c>
+      <c r="C66" t="s">
+        <v>17</v>
+      </c>
+      <c r="D66" t="s">
+        <v>135</v>
+      </c>
+      <c r="E66" t="s">
+        <v>47</v>
+      </c>
+      <c r="F66" t="s">
         <v>136</v>
-      </c>
-      <c r="B66" t="s">
-        <v>137</v>
-      </c>
-      <c r="C66" t="s">
-        <v>13</v>
-      </c>
-      <c r="D66" t="s">
-        <v>140</v>
-      </c>
-      <c r="E66" t="s">
-        <v>139</v>
-      </c>
-      <c r="F66" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>130</v>
+      </c>
+      <c r="B67" t="s">
+        <v>131</v>
+      </c>
+      <c r="C67" t="s">
+        <v>17</v>
+      </c>
+      <c r="D67" t="s">
+        <v>137</v>
+      </c>
+      <c r="E67" t="s">
+        <v>138</v>
+      </c>
+      <c r="F67" t="s">
         <v>136</v>
-      </c>
-      <c r="B67" t="s">
-        <v>137</v>
-      </c>
-      <c r="C67" t="s">
-        <v>17</v>
-      </c>
-      <c r="D67" t="s">
-        <v>141</v>
-      </c>
-      <c r="E67" t="s">
-        <v>47</v>
-      </c>
-      <c r="F67" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B68" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C68" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D68" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="E68" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="F68" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B69" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C69" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D69" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E69" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F69" t="s">
-        <v>147</v>
+        <v>28</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B70" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C70" t="s">
         <v>17</v>
       </c>
       <c r="D70" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="E70" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="F70" t="s">
-        <v>28</v>
+        <v>146</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B71" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C71" t="s">
         <v>17</v>
       </c>
       <c r="D71" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="E71" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="F71" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B72" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C72" t="s">
         <v>17</v>
       </c>
       <c r="D72" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="E72" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="F72" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B73" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C73" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D73" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="E73" t="s">
-        <v>157</v>
+        <v>13</v>
       </c>
       <c r="F73" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B74" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C74" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D74" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E74" t="s">
-        <v>13</v>
+        <v>156</v>
       </c>
       <c r="F74" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B75" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C75" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D75" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E75" t="s">
-        <v>162</v>
+        <v>13</v>
       </c>
       <c r="F75" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B76" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C76" t="s">
         <v>23</v>
       </c>
       <c r="D76" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="E76" t="s">
         <v>13</v>
       </c>
       <c r="F76" t="s">
-        <v>165</v>
+        <v>26</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>136</v>
+        <v>161</v>
       </c>
       <c r="B77" t="s">
-        <v>137</v>
+        <v>13</v>
       </c>
       <c r="C77" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D77" t="s">
-        <v>166</v>
+        <v>18</v>
       </c>
       <c r="E77" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F77" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B78" t="s">
         <v>13</v>
       </c>
       <c r="C78" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D78" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E78" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F78" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="B79" t="s">
         <v>13</v>
       </c>
       <c r="C79" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="D79" t="s">
-        <v>24</v>
+        <v>163</v>
       </c>
       <c r="E79" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F79" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="B80" t="s">
         <v>13</v>
@@ -2416,7 +2398,7 @@
         <v>14</v>
       </c>
       <c r="D80" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="E80" t="s">
         <v>13</v>
@@ -2427,7 +2409,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="B81" t="s">
         <v>13</v>
@@ -2436,7 +2418,7 @@
         <v>14</v>
       </c>
       <c r="D81" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="E81" t="s">
         <v>13</v>
@@ -2447,7 +2429,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="B82" t="s">
         <v>13</v>
@@ -2456,7 +2438,7 @@
         <v>14</v>
       </c>
       <c r="D82" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E82" t="s">
         <v>13</v>
@@ -2467,7 +2449,7 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="B83" t="s">
         <v>13</v>
@@ -2476,7 +2458,7 @@
         <v>14</v>
       </c>
       <c r="D83" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E83" t="s">
         <v>13</v>
@@ -2487,7 +2469,7 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="B84" t="s">
         <v>13</v>
@@ -2496,7 +2478,7 @@
         <v>14</v>
       </c>
       <c r="D84" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="E84" t="s">
         <v>13</v>
@@ -2507,7 +2489,7 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="B85" t="s">
         <v>13</v>
@@ -2516,7 +2498,7 @@
         <v>14</v>
       </c>
       <c r="D85" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="E85" t="s">
         <v>13</v>
@@ -2527,7 +2509,7 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="B86" t="s">
         <v>13</v>
@@ -2536,7 +2518,7 @@
         <v>14</v>
       </c>
       <c r="D86" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="E86" t="s">
         <v>13</v>
@@ -2547,7 +2529,7 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="B87" t="s">
         <v>13</v>
@@ -2556,32 +2538,12 @@
         <v>14</v>
       </c>
       <c r="D87" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="E87" t="s">
         <v>13</v>
       </c>
       <c r="F87" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>168</v>
-      </c>
-      <c r="B88" t="s">
-        <v>13</v>
-      </c>
-      <c r="C88" t="s">
-        <v>14</v>
-      </c>
-      <c r="D88" t="s">
-        <v>177</v>
-      </c>
-      <c r="E88" t="s">
-        <v>13</v>
-      </c>
-      <c r="F88" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
shots: regenerate from the green push run
The referral brief carries the presenter gate and its withheld-mover note, and
the note no longer names anybody the parties block printed.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/e2e/shots/documents/full-report.xlsx
+++ b/dashboard/e2e/shots/documents/full-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="172">
   <si>
     <t>Market intelligence report</t>
   </si>
@@ -181,7 +181,7 @@
     <t>https://www.anaheim.net/DocumentCenter/View/66931/Planning-Commission-Action-Agenda---10202025#item-h6dc7e70418cc</t>
   </si>
   <si>
-    <t>6 further records name the body that brought this matter forward (City of Anaheim; Lisandro Orozco; Stacy Tran). That is who moved it in government rather than who is behind it, so it is not listed above as a party to approach.</t>
+    <t>6 further records name the body that brought this matter forward (City of Anaheim). That is who moved it in government rather than who is behind it, so it is not listed above as a party to approach.</t>
   </si>
   <si>
     <t>2026-02-06. OCVibe Residential Phase I</t>
@@ -289,7 +289,7 @@
     <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/1-23-2026-BOS-Agenda-Packet-FINALcs.pdf#item-6.4-p146</t>
   </si>
   <si>
-    <t>4 further records name the body that brought this matter forward (Craig Sandt, Director of Construction Management; Katherine Luetzow, Director, Planning &amp; Engineering Department: Public Works). That is who moved it in government rather than who is behind it, so it is not listed above as a party to approach.</t>
+    <t>4 further records name the body that brought this matter forward (Katherine Luetzow, Director, Planning &amp; Engineering Department: Public Works; Craig Sandt, Director of Construction Management). That is who moved it in government rather than who is behind it, so it is not listed above as a party to approach.</t>
   </si>
   <si>
     <t>2026-01-01. CFTOD 2045 Comprehensive Plan - recreation / tourist provisions (p.37)</t>
@@ -907,7 +907,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2335,36 +2335,36 @@
         <v>13</v>
       </c>
       <c r="C77" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D77" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E77" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F77" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B78" t="s">
         <v>13</v>
       </c>
       <c r="C78" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="D78" t="s">
-        <v>24</v>
+        <v>163</v>
       </c>
       <c r="E78" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F78" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
@@ -2378,7 +2378,7 @@
         <v>14</v>
       </c>
       <c r="D79" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E79" t="s">
         <v>13</v>
@@ -2398,7 +2398,7 @@
         <v>14</v>
       </c>
       <c r="D80" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E80" t="s">
         <v>13</v>
@@ -2418,7 +2418,7 @@
         <v>14</v>
       </c>
       <c r="D81" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E81" t="s">
         <v>13</v>
@@ -2438,7 +2438,7 @@
         <v>14</v>
       </c>
       <c r="D82" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E82" t="s">
         <v>13</v>
@@ -2458,7 +2458,7 @@
         <v>14</v>
       </c>
       <c r="D83" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E83" t="s">
         <v>13</v>
@@ -2478,7 +2478,7 @@
         <v>14</v>
       </c>
       <c r="D84" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E84" t="s">
         <v>13</v>
@@ -2498,7 +2498,7 @@
         <v>14</v>
       </c>
       <c r="D85" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E85" t="s">
         <v>13</v>
@@ -2518,32 +2518,12 @@
         <v>14</v>
       </c>
       <c r="D86" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E86" t="s">
         <v>13</v>
       </c>
       <c r="F86" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>162</v>
-      </c>
-      <c r="B87" t="s">
-        <v>13</v>
-      </c>
-      <c r="C87" t="s">
-        <v>14</v>
-      </c>
-      <c r="D87" t="s">
-        <v>171</v>
-      </c>
-      <c r="E87" t="s">
-        <v>13</v>
-      </c>
-      <c r="F87" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>